<commit_message>
Build 32: second count labelled Printer fit; Titan kept to the facts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -565,7 +565,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 31 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 32 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -676,12 +676,12 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Titan fit</t>
+          <t>Printer fit</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Titan fit why</t>
+          <t>Printer fit why</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="U24" s="15" t="inlineStr">
         <is>
-          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Titan fit moves from Yes to Partly on that figure.</t>
+          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Printer fit moves from Yes to Partly on that figure.</t>
         </is>
       </c>
       <c r="V24" s="12" t="inlineStr"/>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="U25" s="9" t="inlineStr">
         <is>
-          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Titan fit moves from Yes to Partly on that figure.</t>
+          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Printer fit moves from Yes to Partly on that figure.</t>
         </is>
       </c>
       <c r="V25" s="6" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="U26" s="15" t="inlineStr">
         <is>
-          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Titan fit moves from Yes to Partly on that figure.</t>
+          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Printer fit moves from Yes to Partly on that figure.</t>
         </is>
       </c>
       <c r="V26" s="12" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="U27" s="9" t="inlineStr">
         <is>
-          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Titan fit moves from Yes to Partly on that figure.</t>
+          <t>The 300-closings figure and the even-flow description come from a Builder Magazine profile of 2014 performance. The cadence model is on record; the current volume is not. | Individual profiles for the four named leaders were not found. They are named with titles on the firm's own team page, which is the citation. | The volume on file was more than 300 closings a year. HousingWire reports 973 homes and $310 million in 2025, up 17 percent. Printer fit moves from Yes to Partly on that figure.</t>
         </is>
       </c>
       <c r="V27" s="6" t="inlineStr"/>
@@ -7819,7 +7819,7 @@
       </c>
       <c r="U67" s="9" t="inlineStr">
         <is>
-          <t>The cumulative figure is the firm's own and covers eighteen years. No single-year number is published. | Builder reports 540 closings in 2025 and 552 in 2024. Titan fit moves from Yes to Partly. | No LinkedIn company page exists for the firm, only individual employee profiles.</t>
+          <t>The cumulative figure is the firm's own and covers eighteen years. No single-year number is published. | Builder reports 540 closings in 2025 and 552 in 2024. Printer fit moves from Yes to Partly. | No LinkedIn company page exists for the firm, only individual employee profiles.</t>
         </is>
       </c>
       <c r="V67" s="6" t="inlineStr"/>
@@ -7932,7 +7932,7 @@
       </c>
       <c r="U68" s="15" t="inlineStr">
         <is>
-          <t>The cumulative figure is the firm's own and covers eighteen years. No single-year number is published. | Builder reports 540 closings in 2025 and 552 in 2024. Titan fit moves from Yes to Partly. | No LinkedIn company page exists for the firm, only individual employee profiles.</t>
+          <t>The cumulative figure is the firm's own and covers eighteen years. No single-year number is published. | Builder reports 540 closings in 2025 and 552 in 2024. Printer fit moves from Yes to Partly. | No LinkedIn company page exists for the firm, only individual employee profiles.</t>
         </is>
       </c>
       <c r="V68" s="12" t="inlineStr">
@@ -22195,7 +22195,7 @@
     <row r="197">
       <c r="A197" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both keep a firm in. Only a No takes it out. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 31, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both keep a firm in. Only a No takes it out. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 32, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 36: last sweep, contractor reasons were never rendering
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -565,7 +565,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 35 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 36 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -4814,7 +4814,11 @@
           <t>Spring, Harris-Montgomery</t>
         </is>
       </c>
-      <c r="H42" s="12" t="inlineStr"/>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>No unit count published; owned by Sekisui House U.S.</t>
+        </is>
+      </c>
       <c r="I42" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -4927,7 +4931,11 @@
           <t>Spring, Harris-Montgomery</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr"/>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>No unit count published; owned by Sekisui House U.S.</t>
+        </is>
+      </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -5040,7 +5048,11 @@
           <t>Spring, Harris-Montgomery</t>
         </is>
       </c>
-      <c r="H44" s="12" t="inlineStr"/>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>No unit count published; owned by Sekisui House U.S.</t>
+        </is>
+      </c>
       <c r="I44" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -7033,7 +7045,7 @@
       </c>
       <c r="N61" s="9" t="inlineStr">
         <is>
-          <t>The model is standardisation for entry-level buyers. That is not evidence of paying for an unproven method.</t>
+          <t>The model is standardisation for entry-level buyers. That is not evidence of paying for a method that was new at the time.</t>
         </is>
       </c>
       <c r="O61" s="8" t="inlineStr">
@@ -9469,7 +9481,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>20 homes and $22 million in 2020, the latest published</t>
+          <t>About 75 homes a year on the firm's own count</t>
         </is>
       </c>
       <c r="I83" s="8" t="inlineStr">
@@ -9582,7 +9594,7 @@
       </c>
       <c r="H84" s="12" t="inlineStr">
         <is>
-          <t>20 homes and $22 million in 2020, the latest published</t>
+          <t>About 75 homes a year on the firm's own count</t>
         </is>
       </c>
       <c r="I84" s="14" t="inlineStr">
@@ -9694,7 +9706,7 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>20 homes and $22 million in 2020, the latest published</t>
+          <t>About 75 homes a year on the firm's own count</t>
         </is>
       </c>
       <c r="I85" s="8" t="inlineStr">
@@ -11914,7 +11926,11 @@
           <t>Chicago HQ / Katy, Harris</t>
         </is>
       </c>
-      <c r="H105" s="6" t="inlineStr"/>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>366 build-to-rent units across two Katy projects</t>
+        </is>
+      </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12026,7 +12042,11 @@
           <t>Chicago HQ / Katy, Harris</t>
         </is>
       </c>
-      <c r="H106" s="12" t="inlineStr"/>
+      <c r="H106" s="12" t="inlineStr">
+        <is>
+          <t>366 build-to-rent units across two Katy projects</t>
+        </is>
+      </c>
       <c r="I106" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12142,7 +12162,11 @@
           <t>Chicago HQ / Katy, Harris</t>
         </is>
       </c>
-      <c r="H107" s="6" t="inlineStr"/>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>366 build-to-rent units across two Katy projects</t>
+        </is>
+      </c>
       <c r="I107" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12373,19 +12397,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J109" s="9" t="inlineStr"/>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>The same wall system, installed again and again across Houston and the coast since 2002.</t>
+        </is>
+      </c>
       <c r="K109" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L109" s="9" t="inlineStr"/>
+      <c r="L109" s="9" t="inlineStr">
+        <is>
+          <t>No crew count or homes-a-year figure is published. On the bands, a firm with no published figure is a Partly, and that is the first thing to establish on the call.</t>
+        </is>
+      </c>
       <c r="M109" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N109" s="9" t="inlineStr"/>
+      <c r="N109" s="9" t="inlineStr">
+        <is>
+          <t>Its entire business is a wall method that was new when it adopted it. The crews are trained on twelve form systems and run a twenty-step checklist before every placement.</t>
+        </is>
+      </c>
       <c r="O109" s="8" t="inlineStr">
         <is>
           <t>No</t>
@@ -12469,19 +12505,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J110" s="15" t="inlineStr"/>
+      <c r="J110" s="15" t="inlineStr">
+        <is>
+          <t>Tilt-up and foundation work repeating across four counties from one Houston yard.</t>
+        </is>
+      </c>
       <c r="K110" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L110" s="15" t="inlineStr"/>
+      <c r="L110" s="15" t="inlineStr">
+        <is>
+          <t>150 office and field staff on the firm's own count. That is the only published size in this section, and at that size one or two printers cover a real share of a year's wall.</t>
+        </is>
+      </c>
       <c r="M110" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N110" s="15" t="inlineStr"/>
+      <c r="N110" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record. Its published work is conventional tilt-up and foundations.</t>
+        </is>
+      </c>
       <c r="O110" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12565,19 +12613,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J111" s="9" t="inlineStr"/>
+      <c r="J111" s="9" t="inlineStr">
+        <is>
+          <t>Tilt-up and foundation work repeating across four counties from one Houston yard.</t>
+        </is>
+      </c>
       <c r="K111" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L111" s="9" t="inlineStr"/>
+      <c r="L111" s="9" t="inlineStr">
+        <is>
+          <t>150 office and field staff on the firm's own count. That is the only published size in this section, and at that size one or two printers cover a real share of a year's wall.</t>
+        </is>
+      </c>
       <c r="M111" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N111" s="9" t="inlineStr"/>
+      <c r="N111" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record. Its published work is conventional tilt-up and foundations.</t>
+        </is>
+      </c>
       <c r="O111" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12661,19 +12721,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J112" s="15" t="inlineStr"/>
+      <c r="J112" s="15" t="inlineStr">
+        <is>
+          <t>Tilt-up and foundation work repeating across four counties from one Houston yard.</t>
+        </is>
+      </c>
       <c r="K112" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L112" s="15" t="inlineStr"/>
+      <c r="L112" s="15" t="inlineStr">
+        <is>
+          <t>150 office and field staff on the firm's own count. That is the only published size in this section, and at that size one or two printers cover a real share of a year's wall.</t>
+        </is>
+      </c>
       <c r="M112" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N112" s="15" t="inlineStr"/>
+      <c r="N112" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record. Its published work is conventional tilt-up and foundations.</t>
+        </is>
+      </c>
       <c r="O112" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12753,19 +12825,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J113" s="9" t="inlineStr"/>
+      <c r="J113" s="9" t="inlineStr">
+        <is>
+          <t>Tilt-up warehouses, retail centres and schools repeating inside the Houston market.</t>
+        </is>
+      </c>
       <c r="K113" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L113" s="9" t="inlineStr"/>
+      <c r="L113" s="9" t="inlineStr">
+        <is>
+          <t>No crew count or annual volume is published. The one published job runs to 32 panels across four floors. On the bands, a firm with no annual figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M113" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N113" s="9" t="inlineStr"/>
+      <c r="N113" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record. The 2025 tilt-up award is for execution, not for a new method.</t>
+        </is>
+      </c>
       <c r="O113" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -12838,19 +12922,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J114" s="15" t="inlineStr"/>
+      <c r="J114" s="15" t="inlineStr">
+        <is>
+          <t>Three standing placement divisions in one metro, so the same work recurs rather than arriving one project at a time.</t>
+        </is>
+      </c>
       <c r="K114" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L114" s="15" t="inlineStr"/>
+      <c r="L114" s="15" t="inlineStr">
+        <is>
+          <t>1,500 craftsmen and 975,000 cubic yards a year on the firm's own count. One or two printers would be a line inside the business rather than the business.</t>
+        </is>
+      </c>
       <c r="M114" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N114" s="15" t="inlineStr"/>
+      <c r="N114" s="15" t="inlineStr">
+        <is>
+          <t>It owns a fleet of placing booms and multiple complete hydraulic self-jacking formwork systems on its own account. Buying capital equipment to change how concrete gets placed is the habit this count is looking for, though formwork is not a new method.</t>
+        </is>
+      </c>
       <c r="O114" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12927,19 +13023,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J115" s="9" t="inlineStr"/>
+      <c r="J115" s="9" t="inlineStr">
+        <is>
+          <t>Interior wall and ceiling packages repeating across multifamily and single family work in one metro.</t>
+        </is>
+      </c>
       <c r="K115" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L115" s="9" t="inlineStr"/>
+      <c r="L115" s="9" t="inlineStr">
+        <is>
+          <t>No employee count or annual unit figure is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M115" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N115" s="9" t="inlineStr"/>
+      <c r="N115" s="9" t="inlineStr">
+        <is>
+          <t>It built and staffed a prefabrication plant producing wall panels and interior components offsite, and publishes what that saved on a hospital project. That is paying to move wall work into a factory, which is the nearest thing to the argument for a printer.</t>
+        </is>
+      </c>
       <c r="O115" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13023,19 +13131,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J116" s="15" t="inlineStr"/>
+      <c r="J116" s="15" t="inlineStr">
+        <is>
+          <t>Interior wall and ceiling packages repeating across multifamily and single family work in one metro.</t>
+        </is>
+      </c>
       <c r="K116" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L116" s="15" t="inlineStr"/>
+      <c r="L116" s="15" t="inlineStr">
+        <is>
+          <t>No employee count or annual unit figure is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M116" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N116" s="15" t="inlineStr"/>
+      <c r="N116" s="15" t="inlineStr">
+        <is>
+          <t>It built and staffed a prefabrication plant producing wall panels and interior components offsite, and publishes what that saved on a hospital project. That is paying to move wall work into a factory, which is the nearest thing to the argument for a printer.</t>
+        </is>
+      </c>
       <c r="O116" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13119,19 +13239,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J117" s="9" t="inlineStr"/>
+      <c r="J117" s="9" t="inlineStr">
+        <is>
+          <t>Interior wall and ceiling packages repeating across multifamily and single family work in one metro.</t>
+        </is>
+      </c>
       <c r="K117" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L117" s="9" t="inlineStr"/>
+      <c r="L117" s="9" t="inlineStr">
+        <is>
+          <t>No employee count or annual unit figure is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M117" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N117" s="9" t="inlineStr"/>
+      <c r="N117" s="9" t="inlineStr">
+        <is>
+          <t>It built and staffed a prefabrication plant producing wall panels and interior components offsite, and publishes what that saved on a hospital project. That is paying to move wall work into a factory, which is the nearest thing to the argument for a printer.</t>
+        </is>
+      </c>
       <c r="O117" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13215,19 +13347,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J118" s="15" t="inlineStr"/>
+      <c r="J118" s="15" t="inlineStr">
+        <is>
+          <t>Interior wall and ceiling packages repeating across multifamily and single family work in one metro.</t>
+        </is>
+      </c>
       <c r="K118" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L118" s="15" t="inlineStr"/>
+      <c r="L118" s="15" t="inlineStr">
+        <is>
+          <t>No employee count or annual unit figure is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M118" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N118" s="15" t="inlineStr"/>
+      <c r="N118" s="15" t="inlineStr">
+        <is>
+          <t>It built and staffed a prefabrication plant producing wall panels and interior components offsite, and publishes what that saved on a hospital project. That is paying to move wall work into a factory, which is the nearest thing to the argument for a printer.</t>
+        </is>
+      </c>
       <c r="O118" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13303,19 +13447,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J119" s="9" t="inlineStr"/>
+      <c r="J119" s="9" t="inlineStr">
+        <is>
+          <t>Concrete packages recurring across Houston projects under both delivery models.</t>
+        </is>
+      </c>
       <c r="K119" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L119" s="9" t="inlineStr"/>
+      <c r="L119" s="9" t="inlineStr">
+        <is>
+          <t>No crew count, revenue or project size is published. Nothing on the site sizes the work, so on the bands this is a Partly.</t>
+        </is>
+      </c>
       <c r="M119" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N119" s="9" t="inlineStr"/>
+      <c r="N119" s="9" t="inlineStr">
+        <is>
+          <t>It bought and staffed a modelling stack, Revit, Tekla, AutoCAD and Navisworks, to plan its pours. A printed wall arrives as a model first, so the habit transfers, though modelling is not itself a building method.</t>
+        </is>
+      </c>
       <c r="O119" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -13388,19 +13544,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J120" s="15" t="inlineStr"/>
+      <c r="J120" s="15" t="inlineStr">
+        <is>
+          <t>Design-build projects, each one different.</t>
+        </is>
+      </c>
       <c r="K120" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L120" s="15" t="inlineStr"/>
+      <c r="L120" s="15" t="inlineStr">
+        <is>
+          <t>No headcount, revenue or annual project figure is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M120" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N120" s="15" t="inlineStr"/>
+      <c r="N120" s="15" t="inlineStr">
+        <is>
+          <t>It engineered and delivered a printed house in Houston in collaboration with a printing contractor, and publishes the project on its own site.</t>
+        </is>
+      </c>
       <c r="O120" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -13473,19 +13641,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J121" s="9" t="inlineStr"/>
+      <c r="J121" s="9" t="inlineStr">
+        <is>
+          <t>Commercial buildings across the Gulf Coast. The structures differ project to project.</t>
+        </is>
+      </c>
       <c r="K121" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L121" s="9" t="inlineStr"/>
+      <c r="L121" s="9" t="inlineStr">
+        <is>
+          <t>No revenue, crew count or project count is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M121" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N121" s="9" t="inlineStr"/>
+      <c r="N121" s="9" t="inlineStr">
+        <is>
+          <t>It carries insulated concrete form construction in its standard menu alongside tilt-wall and masonry, so it has sold and built a concrete wall system rather than only a wood one. No named project is published to date it.</t>
+        </is>
+      </c>
       <c r="O121" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -13558,19 +13738,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J122" s="15" t="inlineStr"/>
+      <c r="J122" s="15" t="inlineStr">
+        <is>
+          <t>Industrial and commercial concrete recurring across the east side of the metro.</t>
+        </is>
+      </c>
       <c r="K122" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L122" s="15" t="inlineStr"/>
+      <c r="L122" s="15" t="inlineStr">
+        <is>
+          <t>No crew count, revenue or annual volume is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M122" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N122" s="15" t="inlineStr"/>
+      <c r="N122" s="15" t="inlineStr">
+        <is>
+          <t>It bought volumetric mixers and stood up its own delivery arm rather than buying ready-mix from a plant. That is paying for a different way to get concrete to a site, though it is not a wall method.</t>
+        </is>
+      </c>
       <c r="O122" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -13647,19 +13839,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J123" s="9" t="inlineStr"/>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>Garden-style and mid-rise apartment buildings repeating across Texas markets from a Houston office.</t>
+        </is>
+      </c>
       <c r="K123" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L123" s="9" t="inlineStr"/>
+      <c r="L123" s="9" t="inlineStr">
+        <is>
+          <t>Over 44,000 apartment homes in 45 years, so the wall volume is there. It states that it works through trade partners rather than self-performing, so the machine would sit with a subcontractor rather than with Blazer.</t>
+        </is>
+      </c>
       <c r="M123" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N123" s="9" t="inlineStr"/>
+      <c r="N123" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record. The only construction-method language on the site is the list of building types it builds.</t>
+        </is>
+      </c>
       <c r="O123" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13739,19 +13943,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J124" s="15" t="inlineStr"/>
+      <c r="J124" s="15" t="inlineStr">
+        <is>
+          <t>Garden-style and mid-rise apartment buildings repeating across Texas markets from a Houston office.</t>
+        </is>
+      </c>
       <c r="K124" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L124" s="15" t="inlineStr"/>
+      <c r="L124" s="15" t="inlineStr">
+        <is>
+          <t>Over 44,000 apartment homes in 45 years, so the wall volume is there. It states that it works through trade partners rather than self-performing, so the machine would sit with a subcontractor rather than with Blazer.</t>
+        </is>
+      </c>
       <c r="M124" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N124" s="15" t="inlineStr"/>
+      <c r="N124" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record. The only construction-method language on the site is the list of building types it builds.</t>
+        </is>
+      </c>
       <c r="O124" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13831,19 +14047,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J125" s="9" t="inlineStr"/>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>Garden-style and mid-rise apartment buildings repeating across Texas markets from a Houston office.</t>
+        </is>
+      </c>
       <c r="K125" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L125" s="9" t="inlineStr"/>
+      <c r="L125" s="9" t="inlineStr">
+        <is>
+          <t>Over 44,000 apartment homes in 45 years, so the wall volume is there. It states that it works through trade partners rather than self-performing, so the machine would sit with a subcontractor rather than with Blazer.</t>
+        </is>
+      </c>
       <c r="M125" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N125" s="9" t="inlineStr"/>
+      <c r="N125" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record. The only construction-method language on the site is the list of building types it builds.</t>
+        </is>
+      </c>
       <c r="O125" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13923,19 +14151,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J126" s="15" t="inlineStr"/>
+      <c r="J126" s="15" t="inlineStr">
+        <is>
+          <t>Garden-style and mid-rise apartment buildings repeating across Texas markets from a Houston office.</t>
+        </is>
+      </c>
       <c r="K126" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L126" s="15" t="inlineStr"/>
+      <c r="L126" s="15" t="inlineStr">
+        <is>
+          <t>Over 44,000 apartment homes in 45 years, so the wall volume is there. It states that it works through trade partners rather than self-performing, so the machine would sit with a subcontractor rather than with Blazer.</t>
+        </is>
+      </c>
       <c r="M126" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N126" s="15" t="inlineStr"/>
+      <c r="N126" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record. The only construction-method language on the site is the list of building types it builds.</t>
+        </is>
+      </c>
       <c r="O126" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14015,19 +14255,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J127" s="9" t="inlineStr"/>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>Panel production at the top of the metro's range, recurring across institutional and commercial work.</t>
+        </is>
+      </c>
       <c r="K127" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L127" s="9" t="inlineStr"/>
+      <c r="L127" s="9" t="inlineStr">
+        <is>
+          <t>The concrete business is large enough that a printer is a line item, and the capital decision sits with a listed parent rather than in Houston.</t>
+        </is>
+      </c>
       <c r="M127" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N127" s="9" t="inlineStr"/>
+      <c r="N127" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O127" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14107,19 +14359,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J128" s="15" t="inlineStr"/>
+      <c r="J128" s="15" t="inlineStr">
+        <is>
+          <t>Site and concrete packages recurring across Houston jobs, though the buildings themselves differ.</t>
+        </is>
+      </c>
       <c r="K128" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L128" s="15" t="inlineStr"/>
+      <c r="L128" s="15" t="inlineStr">
+        <is>
+          <t>No crew count, revenue or annual volume is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M128" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N128" s="15" t="inlineStr"/>
+      <c r="N128" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O128" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14192,19 +14456,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J129" s="9" t="inlineStr"/>
+      <c r="J129" s="9" t="inlineStr">
+        <is>
+          <t>Panel and deck work recurring across Houston projects for a standing set of general contractors.</t>
+        </is>
+      </c>
       <c r="K129" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L129" s="9" t="inlineStr"/>
+      <c r="L129" s="9" t="inlineStr">
+        <is>
+          <t>No crew count or annual volume is published. The one published job runs to 49 panels. On the bands, a firm with no annual figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M129" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N129" s="9" t="inlineStr"/>
+      <c r="N129" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O129" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14277,19 +14553,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J130" s="15" t="inlineStr"/>
+      <c r="J130" s="15" t="inlineStr">
+        <is>
+          <t>Commercial shells and paving across the metro. The published square footages are weighted to paving rather than to wall.</t>
+        </is>
+      </c>
       <c r="K130" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L130" s="15" t="inlineStr"/>
+      <c r="L130" s="15" t="inlineStr">
+        <is>
+          <t>No annual volume is published. The one published wall figure is 12,000 square feet of tilt wall against 155,000 gross square feet of paving on the same job.</t>
+        </is>
+      </c>
       <c r="M130" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N130" s="15" t="inlineStr"/>
+      <c r="N130" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O130" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14362,19 +14650,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J131" s="9" t="inlineStr"/>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>Tilt-up buildings recurring across two Texas metros since 1991.</t>
+        </is>
+      </c>
       <c r="K131" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L131" s="9" t="inlineStr"/>
+      <c r="L131" s="9" t="inlineStr">
+        <is>
+          <t>Its own pages carry two different completed square footage figures and neither is repeated here, so nothing published sizes a year's work. On the bands that is a Partly.</t>
+        </is>
+      </c>
       <c r="M131" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N131" s="9" t="inlineStr"/>
+      <c r="N131" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O131" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14451,19 +14751,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J132" s="15" t="inlineStr"/>
+      <c r="J132" s="15" t="inlineStr">
+        <is>
+          <t>Commercial concrete and metal buildings recurring across the north side of the metro.</t>
+        </is>
+      </c>
       <c r="K132" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L132" s="15" t="inlineStr"/>
+      <c r="L132" s="15" t="inlineStr">
+        <is>
+          <t>No crew count, revenue or project size is published anywhere on the site. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M132" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N132" s="15" t="inlineStr"/>
+      <c r="N132" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O132" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14543,19 +14855,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J133" s="9" t="inlineStr"/>
+      <c r="J133" s="9" t="inlineStr">
+        <is>
+          <t>Tilt-up panel production repeats inside one metro even when the buildings differ.</t>
+        </is>
+      </c>
       <c r="K133" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L133" s="9" t="inlineStr"/>
+      <c r="L133" s="9" t="inlineStr">
+        <is>
+          <t>The firm's own site gives a job range of $500,000 to $15 million. A printer would be one line in a book that size.</t>
+        </is>
+      </c>
       <c r="M133" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N133" s="9" t="inlineStr"/>
+      <c r="N133" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record. Its published involvement is in concrete standards committees, not in new methods.</t>
+        </is>
+      </c>
       <c r="O133" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14628,19 +14952,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J134" s="15" t="inlineStr"/>
+      <c r="J134" s="15" t="inlineStr">
+        <is>
+          <t>Panel and structural concrete work recurring across the Houston market.</t>
+        </is>
+      </c>
       <c r="K134" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L134" s="15" t="inlineStr"/>
+      <c r="L134" s="15" t="inlineStr">
+        <is>
+          <t>More than 12,500 people across the United States on the firm's own count, and first on a national ranking of concrete specialty contractors. A machine purchase at that size runs through a national desk, which the bands score as a No.</t>
+        </is>
+      </c>
       <c r="M134" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N134" s="15" t="inlineStr"/>
+      <c r="N134" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record. Working at the top of the panel size range is difficulty, not a new method.</t>
+        </is>
+      </c>
       <c r="O134" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14713,19 +15049,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J135" s="9" t="inlineStr"/>
+      <c r="J135" s="9" t="inlineStr">
+        <is>
+          <t>Single family and townhome communities across the north and west of the metro, taking the same wall package community after community.</t>
+        </is>
+      </c>
       <c r="K135" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L135" s="9" t="inlineStr"/>
+      <c r="L135" s="9" t="inlineStr">
+        <is>
+          <t>9,900 homes a year on the firm's own count, company-wide across Florida and Texas, far above what one or two printers cover. It also counts more than 900 subcontractors and no direct field crew, so there is nobody inside the firm to put on a machine.</t>
+        </is>
+      </c>
       <c r="M135" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N135" s="9" t="inlineStr"/>
+      <c r="N135" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record.</t>
+        </is>
+      </c>
       <c r="O135" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -14802,19 +15150,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J136" s="15" t="inlineStr"/>
+      <c r="J136" s="15" t="inlineStr">
+        <is>
+          <t>Eight divisions across commercial, retail, healthcare and multifamily. The buildings differ project to project.</t>
+        </is>
+      </c>
       <c r="K136" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L136" s="15" t="inlineStr"/>
+      <c r="L136" s="15" t="inlineStr">
+        <is>
+          <t>No annual volume is published. The one published job runs to 770,640 square feet, and the panels on it were poured by somebody else.</t>
+        </is>
+      </c>
       <c r="M136" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N136" s="15" t="inlineStr"/>
+      <c r="N136" s="15" t="inlineStr">
+        <is>
+          <t>It reordered the standard tilt-wall sequence on a 770,640 square foot job, setting a 275-ton lattice boom crane on the perimeter to avoid the slab, and published the result. That is method appetite rather than the purchase of a new method.</t>
+        </is>
+      </c>
       <c r="O136" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14898,19 +15258,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J137" s="9" t="inlineStr"/>
+      <c r="J137" s="9" t="inlineStr">
+        <is>
+          <t>Eight divisions across commercial, retail, healthcare and multifamily. The buildings differ project to project.</t>
+        </is>
+      </c>
       <c r="K137" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L137" s="9" t="inlineStr"/>
+      <c r="L137" s="9" t="inlineStr">
+        <is>
+          <t>No annual volume is published. The one published job runs to 770,640 square feet, and the panels on it were poured by somebody else.</t>
+        </is>
+      </c>
       <c r="M137" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N137" s="9" t="inlineStr"/>
+      <c r="N137" s="9" t="inlineStr">
+        <is>
+          <t>It reordered the standard tilt-wall sequence on a 770,640 square foot job, setting a 275-ton lattice boom crane on the perimeter to avoid the slab, and published the result. That is method appetite rather than the purchase of a new method.</t>
+        </is>
+      </c>
       <c r="O137" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14994,19 +15366,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J138" s="15" t="inlineStr"/>
+      <c r="J138" s="15" t="inlineStr">
+        <is>
+          <t>Eight divisions across commercial, retail, healthcare and multifamily. The buildings differ project to project.</t>
+        </is>
+      </c>
       <c r="K138" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L138" s="15" t="inlineStr"/>
+      <c r="L138" s="15" t="inlineStr">
+        <is>
+          <t>No annual volume is published. The one published job runs to 770,640 square feet, and the panels on it were poured by somebody else.</t>
+        </is>
+      </c>
       <c r="M138" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="N138" s="15" t="inlineStr"/>
+      <c r="N138" s="15" t="inlineStr">
+        <is>
+          <t>It reordered the standard tilt-wall sequence on a 770,640 square foot job, setting a 275-ton lattice boom crane on the perimeter to avoid the slab, and published the result. That is method appetite rather than the purchase of a new method.</t>
+        </is>
+      </c>
       <c r="O138" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -15082,19 +15466,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J139" s="9" t="inlineStr"/>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>Commercial and institutional work rather than a repeated plan, so the structure changes project to project.</t>
+        </is>
+      </c>
       <c r="K139" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L139" s="9" t="inlineStr"/>
+      <c r="L139" s="9" t="inlineStr">
+        <is>
+          <t>No crew count, revenue or annual volume is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M139" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N139" s="9" t="inlineStr"/>
+      <c r="N139" s="9" t="inlineStr">
+        <is>
+          <t>No method statement on record. Owning the equipment and the crews is not the same as having paid for a method that was new at the time.</t>
+        </is>
+      </c>
       <c r="O139" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -15171,19 +15567,31 @@
           <t>Partly</t>
         </is>
       </c>
-      <c r="J140" s="15" t="inlineStr"/>
+      <c r="J140" s="15" t="inlineStr">
+        <is>
+          <t>Commercial and multifamily work across four metros. The buildings differ project to project.</t>
+        </is>
+      </c>
       <c r="K140" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="L140" s="15" t="inlineStr"/>
+      <c r="L140" s="15" t="inlineStr">
+        <is>
+          <t>No revenue, crew count or project size is published. On the bands, a firm with no published figure is a Partly.</t>
+        </is>
+      </c>
       <c r="M140" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N140" s="15" t="inlineStr"/>
+      <c r="N140" s="15" t="inlineStr">
+        <is>
+          <t>No method statement on record. The tilt-up award is for execution.</t>
+        </is>
+      </c>
       <c r="O140" s="14" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -15319,7 +15727,7 @@
       </c>
       <c r="U141" s="9" t="inlineStr">
         <is>
-          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG.  | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
+          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG. | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
         </is>
       </c>
       <c r="V141" s="6" t="inlineStr"/>
@@ -15436,7 +15844,7 @@
       </c>
       <c r="U142" s="15" t="inlineStr">
         <is>
-          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG.  | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
+          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG. | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
         </is>
       </c>
       <c r="V142" s="12" t="inlineStr"/>
@@ -15553,7 +15961,7 @@
       </c>
       <c r="U143" s="9" t="inlineStr">
         <is>
-          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG.  | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
+          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG. | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
         </is>
       </c>
       <c r="V143" s="6" t="inlineStr"/>
@@ -15669,7 +16077,7 @@
       </c>
       <c r="U144" s="15" t="inlineStr">
         <is>
-          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG.  | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
+          <t>The Mill square footage and unit count cross-checked across two sources with differing detail. Treat figures as approximate. | The Mill is the hybrid precedent. A 75,000 square foot six-storey office frame in cross-laminated timber, reported as one of Houston's first, alongside 340 apartments and a 14,000 square foot 1890s brick building kept and folded into the new structure. Michael Hsu and EDI on design. One team ran an unproven structural system and an adaptive reuse on the same six-acre site. | Triten and Radom Capital are the same pair across the Heights packing-plant cluster, M-K-T and the Swift BLDG. | Triten's construction staff below Larry Sloan are construction managers. A Chief Construction Officer is titled to Triten Corporation, a separate Houston company sharing the name. The relationship between the two is unresolved. | No capital signal carries a dollar figure. M-K-T Heights price undisclosed. | LinkedIn URLs unsourced for all four principals.</t>
         </is>
       </c>
       <c r="V144" s="12" t="inlineStr"/>
@@ -22473,7 +22881,11 @@
           <t>Houston / Katy, Harris-Waller</t>
         </is>
       </c>
-      <c r="H203" s="6" t="inlineStr"/>
+      <c r="H203" s="6" t="inlineStr">
+        <is>
+          <t>Sunterra, 2,303 acres in Katy, fifteen builders</t>
+        </is>
+      </c>
       <c r="I203" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -22573,7 +22985,11 @@
           <t>Houston / Katy, Harris-Waller</t>
         </is>
       </c>
-      <c r="H204" s="12" t="inlineStr"/>
+      <c r="H204" s="12" t="inlineStr">
+        <is>
+          <t>Sunterra, 2,303 acres in Katy, fifteen builders</t>
+        </is>
+      </c>
       <c r="I204" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -22673,7 +23089,11 @@
           <t>Cypress / Montgomery, Harris</t>
         </is>
       </c>
-      <c r="H205" s="6" t="inlineStr"/>
+      <c r="H205" s="6" t="inlineStr">
+        <is>
+          <t>Towne Lake and The Highlands, about 4,000 homes</t>
+        </is>
+      </c>
       <c r="I205" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -22777,7 +23197,11 @@
           <t>Houston / Fort Bend, Montgomery</t>
         </is>
       </c>
-      <c r="H206" s="12" t="inlineStr"/>
+      <c r="H206" s="12" t="inlineStr">
+        <is>
+          <t>Fourteen concurrent Houston masterplans</t>
+        </is>
+      </c>
       <c r="I206" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -22881,7 +23305,11 @@
           <t>San Diego HQ / Katy, Harris</t>
         </is>
       </c>
-      <c r="H207" s="6" t="inlineStr"/>
+      <c r="H207" s="6" t="inlineStr">
+        <is>
+          <t>Elyson, 3,600 acres in Katy</t>
+        </is>
+      </c>
       <c r="I207" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -23090,7 +23518,11 @@
           <t>Houston / Montgomery, Galveston</t>
         </is>
       </c>
-      <c r="H209" s="6" t="inlineStr"/>
+      <c r="H209" s="6" t="inlineStr">
+        <is>
+          <t>Sells lots inside its own masterplans; Lennar builds</t>
+        </is>
+      </c>
       <c r="I209" s="8" t="inlineStr">
         <is>
           <t>Partly</t>
@@ -26570,7 +27002,7 @@
     <row r="243">
       <c r="A243" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 35, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 36, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 40: press layer, 32 dated items across 11 firms
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$6:$Z$267</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$6:$AA$267</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z269"/>
+  <dimension ref="A1:AA269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -553,6 +553,7 @@
     <col width="46" customWidth="1" min="24" max="24"/>
     <col width="42" customWidth="1" min="25" max="25"/>
     <col width="42" customWidth="1" min="26" max="26"/>
+    <col width="70" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -565,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 39 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 40 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -754,6 +755,11 @@
           <t>Leadership page</t>
         </is>
       </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>Latest press</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -874,6 +880,11 @@
           <t>https://colekleinbuilders.com/about/</t>
         </is>
       </c>
+      <c r="AA7" s="6" t="inlineStr">
+        <is>
+          <t>2026-02 The Architect's Newspaper. Zuri Gardens, a 3D-printed Texas community, shows promise for attainable housing  https://www.archpaper.com/2026/02/zuri-gardens-3d-printed-texas-community/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -994,6 +1005,11 @@
           <t>https://colekleinbuilders.com/about/</t>
         </is>
       </c>
+      <c r="AA8" s="12" t="inlineStr">
+        <is>
+          <t>2026-02 The Architect's Newspaper. Zuri Gardens, a 3D-printed Texas community, shows promise for attainable housing  https://www.archpaper.com/2026/02/zuri-gardens-3d-printed-texas-community/</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1106,6 +1122,11 @@
       </c>
       <c r="Y9" s="6" t="inlineStr"/>
       <c r="Z9" s="6" t="inlineStr"/>
+      <c r="AA9" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-30 Intelligent Build.tech. Partnership to develop an innovative 3D-printed residential community  https://www.intelligentbuild.tech/2026/04/30/partnership-to-develop-an-innovative-3d-printed-residential-community/</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -1218,6 +1239,11 @@
       </c>
       <c r="Y10" s="12" t="inlineStr"/>
       <c r="Z10" s="12" t="inlineStr"/>
+      <c r="AA10" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22 Homes.com. Houston's 3D-printed housing push grows with two new developments  https://www.homes.com/news/houstons-3d-printed-housing-push-grows-with-two-new-developments/647676272/</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1335,6 +1361,11 @@
           <t>https://wanbridge.com/leadership/</t>
         </is>
       </c>
+      <c r="AA11" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-25 Houston Chronicle. Why Houston's booming build-to-rent sector could slow  https://www.houstonchronicle.com/business/article/houston-build-to-rent-housing-21293194.php</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -1456,6 +1487,11 @@
           <t>https://wanbridge.com/leadership/</t>
         </is>
       </c>
+      <c r="AA12" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-25 Houston Chronicle. Why Houston's booming build-to-rent sector could slow  https://www.houstonchronicle.com/business/article/houston-build-to-rent-housing-21293194.php</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1577,6 +1613,11 @@
           <t>https://wanbridge.com/leadership/</t>
         </is>
       </c>
+      <c r="AA13" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-25 Houston Chronicle. Why Houston's booming build-to-rent sector could slow  https://www.houstonchronicle.com/business/article/houston-build-to-rent-housing-21293194.php</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1694,6 +1735,7 @@
           <t>https://www.lovettcommercial.com/about</t>
         </is>
       </c>
+      <c r="AA14" s="12" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1807,6 +1849,11 @@
       <c r="X15" s="6" t="inlineStr"/>
       <c r="Y15" s="6" t="inlineStr"/>
       <c r="Z15" s="6" t="inlineStr"/>
+      <c r="AA15" s="6" t="inlineStr">
+        <is>
+          <t>2013-10-30 Boxer Property. Boxer Announces Executive Leadership Changes, which is where the current titles come from and which puts engineering and construction under the president  https://www.boxerproperty.com/blog/roles-responsibilities-evolve-executives/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -1920,6 +1967,11 @@
       <c r="X16" s="12" t="inlineStr"/>
       <c r="Y16" s="12" t="inlineStr"/>
       <c r="Z16" s="12" t="inlineStr"/>
+      <c r="AA16" s="12" t="inlineStr">
+        <is>
+          <t>2013-10-30 Boxer Property. Boxer Announces Executive Leadership Changes, which is where the current titles come from and which puts engineering and construction under the president  https://www.boxerproperty.com/blog/roles-responsibilities-evolve-executives/</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2024,6 +2076,11 @@
       <c r="X17" s="6" t="inlineStr"/>
       <c r="Y17" s="6" t="inlineStr"/>
       <c r="Z17" s="6" t="inlineStr"/>
+      <c r="AA17" s="6" t="inlineStr">
+        <is>
+          <t>2013-10-30 Boxer Property. Boxer Announces Executive Leadership Changes, which is where the current titles come from and which puts engineering and construction under the president  https://www.boxerproperty.com/blog/roles-responsibilities-evolve-executives/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -2128,6 +2185,11 @@
       <c r="X18" s="12" t="inlineStr"/>
       <c r="Y18" s="12" t="inlineStr"/>
       <c r="Z18" s="12" t="inlineStr"/>
+      <c r="AA18" s="12" t="inlineStr">
+        <is>
+          <t>2013-10-30 Boxer Property. Boxer Announces Executive Leadership Changes, which is where the current titles come from and which puts engineering and construction under the president  https://www.boxerproperty.com/blog/roles-responsibilities-evolve-executives/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -2240,6 +2302,7 @@
       </c>
       <c r="Y19" s="6" t="inlineStr"/>
       <c r="Z19" s="6" t="inlineStr"/>
+      <c r="AA19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -2360,6 +2423,7 @@
           <t>https://investors.centurycommunities.com/governance/executive-management/default.aspx</t>
         </is>
       </c>
+      <c r="AA20" s="12" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -2477,6 +2541,7 @@
           <t>https://investors.centurycommunities.com/governance/executive-management/default.aspx</t>
         </is>
       </c>
+      <c r="AA21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -2597,6 +2662,11 @@
           <t>https://www.firstamericahomes.com/about/</t>
         </is>
       </c>
+      <c r="AA22" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-10 CEOWORLD magazine. Danny Signorelli Leads First America Homes Expansion Across Houston and Texas  https://ceoworld.biz/2026/08/10/danny-signorelli-leads-first-america-homes-expansion-across-houston-and-texas/</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -2714,6 +2784,11 @@
           <t>https://www.firstamericahomes.com/about/</t>
         </is>
       </c>
+      <c r="AA23" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-10 CEOWORLD magazine. Danny Signorelli Leads First America Homes Expansion Across Houston and Texas  https://ceoworld.biz/2026/08/10/danny-signorelli-leads-first-america-homes-expansion-across-houston-and-texas/</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -2835,6 +2910,11 @@
           <t>https://www.firstamericahomes.com/about/</t>
         </is>
       </c>
+      <c r="AA24" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-10 CEOWORLD magazine. Danny Signorelli Leads First America Homes Expansion Across Houston and Texas  https://ceoworld.biz/2026/08/10/danny-signorelli-leads-first-america-homes-expansion-across-houston-and-texas/</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -2956,6 +3036,11 @@
           <t>https://www.firstamericahomes.com/about/</t>
         </is>
       </c>
+      <c r="AA25" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-10 CEOWORLD magazine. Danny Signorelli Leads First America Homes Expansion Across Houston and Texas  https://ceoworld.biz/2026/08/10/danny-signorelli-leads-first-america-homes-expansion-across-houston-and-texas/</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -3073,6 +3158,11 @@
           <t>https://www.firstamericahomes.com/about/</t>
         </is>
       </c>
+      <c r="AA26" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-10 CEOWORLD magazine. Danny Signorelli Leads First America Homes Expansion Across Houston and Texas  https://ceoworld.biz/2026/08/10/danny-signorelli-leads-first-america-homes-expansion-across-houston-and-texas/</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -3186,6 +3276,11 @@
       </c>
       <c r="Y27" s="6" t="inlineStr"/>
       <c r="Z27" s="6" t="inlineStr"/>
+      <c r="AA27" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24 Builder Magazine. How Stylecraft Is Building Bigger While Staying Local  https://www.builderonline.com/builder-100/leadership/how-stylecraft-is-building-bigger-while-staying-local/</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
@@ -3302,6 +3397,11 @@
       </c>
       <c r="Y28" s="12" t="inlineStr"/>
       <c r="Z28" s="12" t="inlineStr"/>
+      <c r="AA28" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-24 Builder Magazine. How Stylecraft Is Building Bigger While Staying Local  https://www.builderonline.com/builder-100/leadership/how-stylecraft-is-building-bigger-while-staying-local/</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -3419,6 +3519,11 @@
       </c>
       <c r="Y29" s="6" t="inlineStr"/>
       <c r="Z29" s="6" t="inlineStr"/>
+      <c r="AA29" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24 Builder Magazine. How Stylecraft Is Building Bigger While Staying Local  https://www.builderonline.com/builder-100/leadership/how-stylecraft-is-building-bigger-while-staying-local/</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
@@ -3532,6 +3637,11 @@
       </c>
       <c r="Y30" s="12" t="inlineStr"/>
       <c r="Z30" s="12" t="inlineStr"/>
+      <c r="AA30" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-24 Builder Magazine. How Stylecraft Is Building Bigger While Staying Local  https://www.builderonline.com/builder-100/leadership/how-stylecraft-is-building-bigger-while-staying-local/</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -3640,6 +3750,7 @@
       <c r="X31" s="6" t="inlineStr"/>
       <c r="Y31" s="6" t="inlineStr"/>
       <c r="Z31" s="6" t="inlineStr"/>
+      <c r="AA31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
@@ -3744,6 +3855,7 @@
       <c r="X32" s="12" t="inlineStr"/>
       <c r="Y32" s="12" t="inlineStr"/>
       <c r="Z32" s="12" t="inlineStr"/>
+      <c r="AA32" s="12" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -3848,6 +3960,7 @@
       <c r="X33" s="6" t="inlineStr"/>
       <c r="Y33" s="6" t="inlineStr"/>
       <c r="Z33" s="6" t="inlineStr"/>
+      <c r="AA33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
@@ -3956,6 +4069,7 @@
       <c r="X34" s="12" t="inlineStr"/>
       <c r="Y34" s="12" t="inlineStr"/>
       <c r="Z34" s="12" t="inlineStr"/>
+      <c r="AA34" s="12" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -4076,6 +4190,7 @@
           <t>https://avenuecdc.org/about-us/board-staff/</t>
         </is>
       </c>
+      <c r="AA35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
@@ -4193,6 +4308,7 @@
           <t>https://avenuecdc.org/about-us/board-staff/</t>
         </is>
       </c>
+      <c r="AA36" s="12" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -4310,6 +4426,7 @@
           <t>https://avenuecdc.org/about-us/board-staff/</t>
         </is>
       </c>
+      <c r="AA37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
@@ -4431,6 +4548,7 @@
           <t>https://avenuecdc.org/about-us/board-staff/</t>
         </is>
       </c>
+      <c r="AA38" s="12" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -4548,6 +4666,7 @@
           <t>https://suebausa.com/about-us/</t>
         </is>
       </c>
+      <c r="AA39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
@@ -4668,6 +4787,7 @@
           <t>https://suebausa.com/about-us/</t>
         </is>
       </c>
+      <c r="AA40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -4789,6 +4909,7 @@
           <t>https://suebausa.com/about-us/</t>
         </is>
       </c>
+      <c r="AA41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
@@ -4906,6 +5027,11 @@
         </is>
       </c>
       <c r="Z42" s="12" t="inlineStr"/>
+      <c r="AA42" s="12" t="inlineStr">
+        <is>
+          <t>Builder Magazine. Chesmar Homes, with the note that Sekisui House U.S. is the 2026 Builder of the Year  https://www.builderonline.com/organization/chesmar-homes/</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -5023,6 +5149,11 @@
         </is>
       </c>
       <c r="Z43" s="6" t="inlineStr"/>
+      <c r="AA43" s="6" t="inlineStr">
+        <is>
+          <t>Builder Magazine. Chesmar Homes, with the note that Sekisui House U.S. is the 2026 Builder of the Year  https://www.builderonline.com/organization/chesmar-homes/</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
@@ -5140,6 +5271,11 @@
         </is>
       </c>
       <c r="Z44" s="12" t="inlineStr"/>
+      <c r="AA44" s="12" t="inlineStr">
+        <is>
+          <t>Builder Magazine. Chesmar Homes, with the note that Sekisui House U.S. is the 2026 Builder of the Year  https://www.builderonline.com/organization/chesmar-homes/</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -5252,6 +5388,7 @@
       </c>
       <c r="Y45" s="6" t="inlineStr"/>
       <c r="Z45" s="6" t="inlineStr"/>
+      <c r="AA45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
@@ -5364,6 +5501,7 @@
       </c>
       <c r="Y46" s="12" t="inlineStr"/>
       <c r="Z46" s="12" t="inlineStr"/>
+      <c r="AA46" s="12" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -5476,6 +5614,7 @@
       </c>
       <c r="Y47" s="6" t="inlineStr"/>
       <c r="Z47" s="6" t="inlineStr"/>
+      <c r="AA47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
@@ -5588,6 +5727,7 @@
       </c>
       <c r="Y48" s="12" t="inlineStr"/>
       <c r="Z48" s="12" t="inlineStr"/>
+      <c r="AA48" s="12" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -5704,6 +5844,7 @@
       </c>
       <c r="Y49" s="6" t="inlineStr"/>
       <c r="Z49" s="6" t="inlineStr"/>
+      <c r="AA49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
@@ -5813,6 +5954,7 @@
       <c r="X50" s="12" t="inlineStr"/>
       <c r="Y50" s="12" t="inlineStr"/>
       <c r="Z50" s="12" t="inlineStr"/>
+      <c r="AA50" s="12" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -5926,6 +6068,7 @@
       <c r="X51" s="6" t="inlineStr"/>
       <c r="Y51" s="6" t="inlineStr"/>
       <c r="Z51" s="6" t="inlineStr"/>
+      <c r="AA51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
@@ -6035,6 +6178,7 @@
       <c r="X52" s="12" t="inlineStr"/>
       <c r="Y52" s="12" t="inlineStr"/>
       <c r="Z52" s="12" t="inlineStr"/>
+      <c r="AA52" s="12" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -6155,6 +6299,7 @@
           <t>https://housingforhouston.com/leadership/executive-leadership/</t>
         </is>
       </c>
+      <c r="AA53" s="6" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
@@ -6276,6 +6421,7 @@
           <t>https://housingforhouston.com/leadership/executive-leadership/</t>
         </is>
       </c>
+      <c r="AA54" s="12" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -6393,6 +6539,7 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
+      <c r="AA55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
@@ -6513,6 +6660,7 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
+      <c r="AA56" s="12" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -6633,6 +6781,7 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
+      <c r="AA57" s="6" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
@@ -6754,6 +6903,7 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
+      <c r="AA58" s="12" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -6871,6 +7021,7 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
+      <c r="AA59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
@@ -6988,6 +7139,7 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
+      <c r="AA60" s="12" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -7100,6 +7252,7 @@
       </c>
       <c r="Y61" s="6" t="inlineStr"/>
       <c r="Z61" s="6" t="inlineStr"/>
+      <c r="AA61" s="6" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
@@ -7220,6 +7373,7 @@
           <t>https://www.camillocompanies.com/about-us</t>
         </is>
       </c>
+      <c r="AA62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -7340,6 +7494,7 @@
           <t>https://www.camillocompanies.com/about-us</t>
         </is>
       </c>
+      <c r="AA63" s="6" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -7460,6 +7615,7 @@
           <t>https://www.camillocompanies.com/about-us</t>
         </is>
       </c>
+      <c r="AA64" s="12" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -7580,6 +7736,7 @@
           <t>https://www.camillocompanies.com/about-us</t>
         </is>
       </c>
+      <c r="AA65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
@@ -7700,6 +7857,7 @@
           <t>https://www.c-rock.com/about</t>
         </is>
       </c>
+      <c r="AA66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -7817,6 +7975,7 @@
           <t>https://www.c-rock.com/about</t>
         </is>
       </c>
+      <c r="AA67" s="6" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
@@ -7934,6 +8093,7 @@
           <t>https://www.c-rock.com/about</t>
         </is>
       </c>
+      <c r="AA68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -8054,6 +8214,7 @@
           <t>https://www.christophertodd.com/our-story/</t>
         </is>
       </c>
+      <c r="AA69" s="6" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
@@ -8174,6 +8335,7 @@
           <t>https://www.christophertodd.com/our-story/</t>
         </is>
       </c>
+      <c r="AA70" s="12" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -8282,6 +8444,7 @@
       <c r="X71" s="6" t="inlineStr"/>
       <c r="Y71" s="6" t="inlineStr"/>
       <c r="Z71" s="6" t="inlineStr"/>
+      <c r="AA71" s="6" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
@@ -8390,6 +8553,7 @@
       <c r="X72" s="12" t="inlineStr"/>
       <c r="Y72" s="12" t="inlineStr"/>
       <c r="Z72" s="12" t="inlineStr"/>
+      <c r="AA72" s="12" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -8487,6 +8651,7 @@
       <c r="X73" s="6" t="inlineStr"/>
       <c r="Y73" s="6" t="inlineStr"/>
       <c r="Z73" s="6" t="inlineStr"/>
+      <c r="AA73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
@@ -8595,6 +8760,7 @@
       <c r="X74" s="12" t="inlineStr"/>
       <c r="Y74" s="12" t="inlineStr"/>
       <c r="Z74" s="12" t="inlineStr"/>
+      <c r="AA74" s="12" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -8699,6 +8865,7 @@
       <c r="X75" s="6" t="inlineStr"/>
       <c r="Y75" s="6" t="inlineStr"/>
       <c r="Z75" s="6" t="inlineStr"/>
+      <c r="AA75" s="6" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
@@ -8796,6 +8963,7 @@
       <c r="X76" s="12" t="inlineStr"/>
       <c r="Y76" s="12" t="inlineStr"/>
       <c r="Z76" s="12" t="inlineStr"/>
+      <c r="AA76" s="12" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
@@ -8905,6 +9073,7 @@
       <c r="X77" s="6" t="inlineStr"/>
       <c r="Y77" s="6" t="inlineStr"/>
       <c r="Z77" s="6" t="inlineStr"/>
+      <c r="AA77" s="6" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
@@ -9013,6 +9182,7 @@
       <c r="X78" s="12" t="inlineStr"/>
       <c r="Y78" s="12" t="inlineStr"/>
       <c r="Z78" s="12" t="inlineStr"/>
+      <c r="AA78" s="12" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
@@ -9117,6 +9287,7 @@
       <c r="X79" s="6" t="inlineStr"/>
       <c r="Y79" s="6" t="inlineStr"/>
       <c r="Z79" s="6" t="inlineStr"/>
+      <c r="AA79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
@@ -9229,6 +9400,7 @@
       </c>
       <c r="Y80" s="12" t="inlineStr"/>
       <c r="Z80" s="12" t="inlineStr"/>
+      <c r="AA80" s="12" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -9342,6 +9514,7 @@
       <c r="X81" s="6" t="inlineStr"/>
       <c r="Y81" s="6" t="inlineStr"/>
       <c r="Z81" s="6" t="inlineStr"/>
+      <c r="AA81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
@@ -9454,6 +9627,7 @@
       </c>
       <c r="Y82" s="12" t="inlineStr"/>
       <c r="Z82" s="12" t="inlineStr"/>
+      <c r="AA82" s="12" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -9567,6 +9741,7 @@
       </c>
       <c r="Y83" s="6" t="inlineStr"/>
       <c r="Z83" s="6" t="inlineStr"/>
+      <c r="AA83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
@@ -9679,6 +9854,7 @@
       </c>
       <c r="Y84" s="12" t="inlineStr"/>
       <c r="Z84" s="12" t="inlineStr"/>
+      <c r="AA84" s="12" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -9791,6 +9967,7 @@
       </c>
       <c r="Y85" s="6" t="inlineStr"/>
       <c r="Z85" s="6" t="inlineStr"/>
+      <c r="AA85" s="6" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
@@ -9908,6 +10085,7 @@
       </c>
       <c r="Y86" s="12" t="inlineStr"/>
       <c r="Z86" s="12" t="inlineStr"/>
+      <c r="AA86" s="12" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
@@ -10021,6 +10199,7 @@
       </c>
       <c r="Y87" s="6" t="inlineStr"/>
       <c r="Z87" s="6" t="inlineStr"/>
+      <c r="AA87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
@@ -10125,6 +10304,7 @@
       <c r="X88" s="12" t="inlineStr"/>
       <c r="Y88" s="12" t="inlineStr"/>
       <c r="Z88" s="12" t="inlineStr"/>
+      <c r="AA88" s="12" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
@@ -10229,6 +10409,7 @@
       <c r="X89" s="6" t="inlineStr"/>
       <c r="Y89" s="6" t="inlineStr"/>
       <c r="Z89" s="6" t="inlineStr"/>
+      <c r="AA89" s="6" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
@@ -10342,6 +10523,7 @@
       <c r="X90" s="12" t="inlineStr"/>
       <c r="Y90" s="12" t="inlineStr"/>
       <c r="Z90" s="12" t="inlineStr"/>
+      <c r="AA90" s="12" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
@@ -10462,6 +10644,7 @@
           <t>https://provident.net/our-team/</t>
         </is>
       </c>
+      <c r="AA91" s="6" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
@@ -10582,6 +10765,7 @@
           <t>https://provident.net/our-team/</t>
         </is>
       </c>
+      <c r="AA92" s="12" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
@@ -10695,6 +10879,7 @@
       </c>
       <c r="Y93" s="6" t="inlineStr"/>
       <c r="Z93" s="6" t="inlineStr"/>
+      <c r="AA93" s="6" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
@@ -10808,6 +10993,7 @@
       </c>
       <c r="Y94" s="12" t="inlineStr"/>
       <c r="Z94" s="12" t="inlineStr"/>
+      <c r="AA94" s="12" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
@@ -10921,6 +11107,7 @@
         </is>
       </c>
       <c r="Z95" s="6" t="inlineStr"/>
+      <c r="AA95" s="6" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
@@ -11034,6 +11221,7 @@
         </is>
       </c>
       <c r="Z96" s="12" t="inlineStr"/>
+      <c r="AA96" s="12" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
@@ -11146,6 +11334,7 @@
       </c>
       <c r="Y97" s="6" t="inlineStr"/>
       <c r="Z97" s="6" t="inlineStr"/>
+      <c r="AA97" s="6" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
@@ -11255,6 +11444,7 @@
       <c r="X98" s="12" t="inlineStr"/>
       <c r="Y98" s="12" t="inlineStr"/>
       <c r="Z98" s="12" t="inlineStr"/>
+      <c r="AA98" s="12" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
@@ -11359,6 +11549,7 @@
       <c r="X99" s="6" t="inlineStr"/>
       <c r="Y99" s="6" t="inlineStr"/>
       <c r="Z99" s="6" t="inlineStr"/>
+      <c r="AA99" s="6" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
@@ -11468,6 +11659,7 @@
       <c r="X100" s="12" t="inlineStr"/>
       <c r="Y100" s="12" t="inlineStr"/>
       <c r="Z100" s="12" t="inlineStr"/>
+      <c r="AA100" s="12" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
@@ -11580,6 +11772,7 @@
       </c>
       <c r="Y101" s="6" t="inlineStr"/>
       <c r="Z101" s="6" t="inlineStr"/>
+      <c r="AA101" s="6" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
@@ -11684,6 +11877,7 @@
       <c r="X102" s="12" t="inlineStr"/>
       <c r="Y102" s="12" t="inlineStr"/>
       <c r="Z102" s="12" t="inlineStr"/>
+      <c r="AA102" s="12" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
@@ -11797,6 +11991,7 @@
       <c r="X103" s="6" t="inlineStr"/>
       <c r="Y103" s="6" t="inlineStr"/>
       <c r="Z103" s="6" t="inlineStr"/>
+      <c r="AA103" s="6" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
@@ -11901,6 +12096,7 @@
       <c r="X104" s="12" t="inlineStr"/>
       <c r="Y104" s="12" t="inlineStr"/>
       <c r="Z104" s="12" t="inlineStr"/>
+      <c r="AA104" s="12" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
@@ -12017,6 +12213,7 @@
           <t>https://rskrealestatepartners.com/our-team/</t>
         </is>
       </c>
+      <c r="AA105" s="6" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="12" t="inlineStr">
@@ -12137,6 +12334,7 @@
           <t>https://rskrealestatepartners.com/our-team/</t>
         </is>
       </c>
+      <c r="AA106" s="12" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
@@ -12253,6 +12451,7 @@
           <t>https://rskrealestatepartners.com/our-team/</t>
         </is>
       </c>
+      <c r="AA107" s="6" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="12" t="inlineStr">
@@ -12362,6 +12561,7 @@
       <c r="X108" s="12" t="inlineStr"/>
       <c r="Y108" s="12" t="inlineStr"/>
       <c r="Z108" s="12" t="inlineStr"/>
+      <c r="AA108" s="12" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
@@ -12470,6 +12670,7 @@
       <c r="X109" s="6" t="inlineStr"/>
       <c r="Y109" s="6" t="inlineStr"/>
       <c r="Z109" s="6" t="inlineStr"/>
+      <c r="AA109" s="6" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
@@ -12583,6 +12784,7 @@
       <c r="X110" s="12" t="inlineStr"/>
       <c r="Y110" s="12" t="inlineStr"/>
       <c r="Z110" s="12" t="inlineStr"/>
+      <c r="AA110" s="12" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
@@ -12696,6 +12898,7 @@
       <c r="X111" s="6" t="inlineStr"/>
       <c r="Y111" s="6" t="inlineStr"/>
       <c r="Z111" s="6" t="inlineStr"/>
+      <c r="AA111" s="6" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
@@ -12804,6 +13007,7 @@
       <c r="X112" s="12" t="inlineStr"/>
       <c r="Y112" s="12" t="inlineStr"/>
       <c r="Z112" s="12" t="inlineStr"/>
+      <c r="AA112" s="12" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
@@ -12917,6 +13121,7 @@
       <c r="X113" s="6" t="inlineStr"/>
       <c r="Y113" s="6" t="inlineStr"/>
       <c r="Z113" s="6" t="inlineStr"/>
+      <c r="AA113" s="6" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="12" t="inlineStr">
@@ -13030,6 +13235,7 @@
       <c r="X114" s="12" t="inlineStr"/>
       <c r="Y114" s="12" t="inlineStr"/>
       <c r="Z114" s="12" t="inlineStr"/>
+      <c r="AA114" s="12" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
@@ -13143,6 +13349,7 @@
       <c r="X115" s="6" t="inlineStr"/>
       <c r="Y115" s="6" t="inlineStr"/>
       <c r="Z115" s="6" t="inlineStr"/>
+      <c r="AA115" s="6" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
@@ -13256,6 +13463,7 @@
       <c r="X116" s="12" t="inlineStr"/>
       <c r="Y116" s="12" t="inlineStr"/>
       <c r="Z116" s="12" t="inlineStr"/>
+      <c r="AA116" s="12" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
@@ -13369,6 +13577,7 @@
       <c r="X117" s="6" t="inlineStr"/>
       <c r="Y117" s="6" t="inlineStr"/>
       <c r="Z117" s="6" t="inlineStr"/>
+      <c r="AA117" s="6" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
@@ -13477,6 +13686,7 @@
       <c r="X118" s="12" t="inlineStr"/>
       <c r="Y118" s="12" t="inlineStr"/>
       <c r="Z118" s="12" t="inlineStr"/>
+      <c r="AA118" s="12" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
@@ -13585,6 +13795,7 @@
       <c r="X119" s="6" t="inlineStr"/>
       <c r="Y119" s="6" t="inlineStr"/>
       <c r="Z119" s="6" t="inlineStr"/>
+      <c r="AA119" s="6" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
@@ -13689,6 +13900,7 @@
       <c r="X120" s="12" t="inlineStr"/>
       <c r="Y120" s="12" t="inlineStr"/>
       <c r="Z120" s="12" t="inlineStr"/>
+      <c r="AA120" s="12" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
@@ -13802,6 +14014,7 @@
       <c r="X121" s="6" t="inlineStr"/>
       <c r="Y121" s="6" t="inlineStr"/>
       <c r="Z121" s="6" t="inlineStr"/>
+      <c r="AA121" s="6" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
@@ -13915,6 +14128,7 @@
       <c r="X122" s="12" t="inlineStr"/>
       <c r="Y122" s="12" t="inlineStr"/>
       <c r="Z122" s="12" t="inlineStr"/>
+      <c r="AA122" s="12" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
@@ -14024,6 +14238,7 @@
       <c r="X123" s="6" t="inlineStr"/>
       <c r="Y123" s="6" t="inlineStr"/>
       <c r="Z123" s="6" t="inlineStr"/>
+      <c r="AA123" s="6" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
@@ -14137,6 +14352,11 @@
       <c r="X124" s="12" t="inlineStr"/>
       <c r="Y124" s="12" t="inlineStr"/>
       <c r="Z124" s="12" t="inlineStr"/>
+      <c r="AA124" s="12" t="inlineStr">
+        <is>
+          <t>2025-03 Construction In Focus. CIVE, Construction and Design at their Finest  https://constructioninfocus.com/2025/03/cive-construction-and-design-at-their-finest/</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
@@ -14250,6 +14470,11 @@
       <c r="X125" s="6" t="inlineStr"/>
       <c r="Y125" s="6" t="inlineStr"/>
       <c r="Z125" s="6" t="inlineStr"/>
+      <c r="AA125" s="6" t="inlineStr">
+        <is>
+          <t>2025-03 Construction In Focus. CIVE, Construction and Design at their Finest  https://constructioninfocus.com/2025/03/cive-construction-and-design-at-their-finest/</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
@@ -14358,6 +14583,11 @@
       <c r="X126" s="12" t="inlineStr"/>
       <c r="Y126" s="12" t="inlineStr"/>
       <c r="Z126" s="12" t="inlineStr"/>
+      <c r="AA126" s="12" t="inlineStr">
+        <is>
+          <t>2025-03 Construction In Focus. CIVE, Construction and Design at their Finest  https://constructioninfocus.com/2025/03/cive-construction-and-design-at-their-finest/</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
@@ -14471,6 +14701,7 @@
       <c r="X127" s="6" t="inlineStr"/>
       <c r="Y127" s="6" t="inlineStr"/>
       <c r="Z127" s="6" t="inlineStr"/>
+      <c r="AA127" s="6" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
@@ -14584,6 +14815,7 @@
       <c r="X128" s="12" t="inlineStr"/>
       <c r="Y128" s="12" t="inlineStr"/>
       <c r="Z128" s="12" t="inlineStr"/>
+      <c r="AA128" s="12" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
@@ -14688,6 +14920,7 @@
       <c r="X129" s="6" t="inlineStr"/>
       <c r="Y129" s="6" t="inlineStr"/>
       <c r="Z129" s="6" t="inlineStr"/>
+      <c r="AA129" s="6" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="12" t="inlineStr">
@@ -14792,6 +15025,7 @@
       <c r="X130" s="12" t="inlineStr"/>
       <c r="Y130" s="12" t="inlineStr"/>
       <c r="Z130" s="12" t="inlineStr"/>
+      <c r="AA130" s="12" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
@@ -14896,6 +15130,7 @@
       <c r="X131" s="6" t="inlineStr"/>
       <c r="Y131" s="6" t="inlineStr"/>
       <c r="Z131" s="6" t="inlineStr"/>
+      <c r="AA131" s="6" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
@@ -15000,6 +15235,7 @@
       <c r="X132" s="12" t="inlineStr"/>
       <c r="Y132" s="12" t="inlineStr"/>
       <c r="Z132" s="12" t="inlineStr"/>
+      <c r="AA132" s="12" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
@@ -15104,6 +15340,7 @@
       <c r="X133" s="6" t="inlineStr"/>
       <c r="Y133" s="6" t="inlineStr"/>
       <c r="Z133" s="6" t="inlineStr"/>
+      <c r="AA133" s="6" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
@@ -15208,6 +15445,7 @@
       <c r="X134" s="12" t="inlineStr"/>
       <c r="Y134" s="12" t="inlineStr"/>
       <c r="Z134" s="12" t="inlineStr"/>
+      <c r="AA134" s="12" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
@@ -15312,6 +15550,7 @@
       <c r="X135" s="6" t="inlineStr"/>
       <c r="Y135" s="6" t="inlineStr"/>
       <c r="Z135" s="6" t="inlineStr"/>
+      <c r="AA135" s="6" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
@@ -15420,6 +15659,7 @@
       <c r="X136" s="12" t="inlineStr"/>
       <c r="Y136" s="12" t="inlineStr"/>
       <c r="Z136" s="12" t="inlineStr"/>
+      <c r="AA136" s="12" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
@@ -15524,6 +15764,7 @@
       <c r="X137" s="6" t="inlineStr"/>
       <c r="Y137" s="6" t="inlineStr"/>
       <c r="Z137" s="6" t="inlineStr"/>
+      <c r="AA137" s="6" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
@@ -15633,6 +15874,7 @@
       <c r="X138" s="12" t="inlineStr"/>
       <c r="Y138" s="12" t="inlineStr"/>
       <c r="Z138" s="12" t="inlineStr"/>
+      <c r="AA138" s="12" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
@@ -15742,6 +15984,7 @@
       <c r="X139" s="6" t="inlineStr"/>
       <c r="Y139" s="6" t="inlineStr"/>
       <c r="Z139" s="6" t="inlineStr"/>
+      <c r="AA139" s="6" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
@@ -15846,6 +16089,11 @@
       <c r="X140" s="12" t="inlineStr"/>
       <c r="Y140" s="12" t="inlineStr"/>
       <c r="Z140" s="12" t="inlineStr"/>
+      <c r="AA140" s="12" t="inlineStr">
+        <is>
+          <t>2026 Engineering News-Record. ENR 2026 Top 400 Contractors, where the firm is ranked 72  https://www.enr.com/toplists/2026-Top-400-Contractors-1</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
@@ -15950,6 +16198,11 @@
       <c r="X141" s="6" t="inlineStr"/>
       <c r="Y141" s="6" t="inlineStr"/>
       <c r="Z141" s="6" t="inlineStr"/>
+      <c r="AA141" s="6" t="inlineStr">
+        <is>
+          <t>2026 Engineering News-Record. ENR 2026 Top 400 Contractors, where the firm is ranked 72  https://www.enr.com/toplists/2026-Top-400-Contractors-1</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
@@ -16054,6 +16307,11 @@
       <c r="X142" s="12" t="inlineStr"/>
       <c r="Y142" s="12" t="inlineStr"/>
       <c r="Z142" s="12" t="inlineStr"/>
+      <c r="AA142" s="12" t="inlineStr">
+        <is>
+          <t>2026 Engineering News-Record. ENR 2026 Top 400 Contractors, where the firm is ranked 72  https://www.enr.com/toplists/2026-Top-400-Contractors-1</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
@@ -16167,6 +16425,11 @@
       <c r="X143" s="6" t="inlineStr"/>
       <c r="Y143" s="6" t="inlineStr"/>
       <c r="Z143" s="6" t="inlineStr"/>
+      <c r="AA143" s="6" t="inlineStr">
+        <is>
+          <t>2026 Engineering News-Record. ENR 2026 Top 400 Contractors, where the firm is ranked 72  https://www.enr.com/toplists/2026-Top-400-Contractors-1</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
@@ -16276,6 +16539,11 @@
       <c r="X144" s="12" t="inlineStr"/>
       <c r="Y144" s="12" t="inlineStr"/>
       <c r="Z144" s="12" t="inlineStr"/>
+      <c r="AA144" s="12" t="inlineStr">
+        <is>
+          <t>2026 Engineering News-Record. ENR 2026 Top 400 Contractors, where the firm is ranked 72  https://www.enr.com/toplists/2026-Top-400-Contractors-1</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
@@ -16384,6 +16652,7 @@
       <c r="X145" s="6" t="inlineStr"/>
       <c r="Y145" s="6" t="inlineStr"/>
       <c r="Z145" s="6" t="inlineStr"/>
+      <c r="AA145" s="6" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
@@ -16488,6 +16757,7 @@
       <c r="X146" s="12" t="inlineStr"/>
       <c r="Y146" s="12" t="inlineStr"/>
       <c r="Z146" s="12" t="inlineStr"/>
+      <c r="AA146" s="12" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
@@ -16597,6 +16867,7 @@
       <c r="X147" s="6" t="inlineStr"/>
       <c r="Y147" s="6" t="inlineStr"/>
       <c r="Z147" s="6" t="inlineStr"/>
+      <c r="AA147" s="6" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
@@ -16706,6 +16977,7 @@
       <c r="X148" s="12" t="inlineStr"/>
       <c r="Y148" s="12" t="inlineStr"/>
       <c r="Z148" s="12" t="inlineStr"/>
+      <c r="AA148" s="12" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
@@ -16815,6 +17087,7 @@
       <c r="X149" s="6" t="inlineStr"/>
       <c r="Y149" s="6" t="inlineStr"/>
       <c r="Z149" s="6" t="inlineStr"/>
+      <c r="AA149" s="6" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
@@ -16924,6 +17197,7 @@
       <c r="X150" s="12" t="inlineStr"/>
       <c r="Y150" s="12" t="inlineStr"/>
       <c r="Z150" s="12" t="inlineStr"/>
+      <c r="AA150" s="12" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
@@ -17028,6 +17302,7 @@
       <c r="X151" s="6" t="inlineStr"/>
       <c r="Y151" s="6" t="inlineStr"/>
       <c r="Z151" s="6" t="inlineStr"/>
+      <c r="AA151" s="6" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="12" t="inlineStr">
@@ -17132,6 +17407,7 @@
       <c r="X152" s="12" t="inlineStr"/>
       <c r="Y152" s="12" t="inlineStr"/>
       <c r="Z152" s="12" t="inlineStr"/>
+      <c r="AA152" s="12" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
@@ -17236,6 +17512,7 @@
       <c r="X153" s="6" t="inlineStr"/>
       <c r="Y153" s="6" t="inlineStr"/>
       <c r="Z153" s="6" t="inlineStr"/>
+      <c r="AA153" s="6" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="12" t="inlineStr">
@@ -17345,6 +17622,7 @@
       <c r="X154" s="12" t="inlineStr"/>
       <c r="Y154" s="12" t="inlineStr"/>
       <c r="Z154" s="12" t="inlineStr"/>
+      <c r="AA154" s="12" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
@@ -17454,6 +17732,7 @@
       <c r="X155" s="6" t="inlineStr"/>
       <c r="Y155" s="6" t="inlineStr"/>
       <c r="Z155" s="6" t="inlineStr"/>
+      <c r="AA155" s="6" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="12" t="inlineStr">
@@ -17562,6 +17841,7 @@
       <c r="X156" s="12" t="inlineStr"/>
       <c r="Y156" s="12" t="inlineStr"/>
       <c r="Z156" s="12" t="inlineStr"/>
+      <c r="AA156" s="12" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
@@ -17675,6 +17955,7 @@
       <c r="X157" s="6" t="inlineStr"/>
       <c r="Y157" s="6" t="inlineStr"/>
       <c r="Z157" s="6" t="inlineStr"/>
+      <c r="AA157" s="6" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="12" t="inlineStr">
@@ -17772,6 +18053,7 @@
       <c r="X158" s="12" t="inlineStr"/>
       <c r="Y158" s="12" t="inlineStr"/>
       <c r="Z158" s="12" t="inlineStr"/>
+      <c r="AA158" s="12" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="6" t="inlineStr">
@@ -17881,6 +18163,7 @@
       <c r="X159" s="6" t="inlineStr"/>
       <c r="Y159" s="6" t="inlineStr"/>
       <c r="Z159" s="6" t="inlineStr"/>
+      <c r="AA159" s="6" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="12" t="inlineStr">
@@ -17994,6 +18277,11 @@
       <c r="X160" s="12" t="inlineStr"/>
       <c r="Y160" s="12" t="inlineStr"/>
       <c r="Z160" s="12" t="inlineStr"/>
+      <c r="AA160" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-21 Construction Owners. Arch-Con Tops Out 330-Unit Artis Montrose Apartment Project  https://www.constructionowners.com/news/arch-con-reaches-topping-out-milestone-on-330-unit-artis-montrose-apartment-project</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
@@ -18102,6 +18390,11 @@
       <c r="X161" s="6" t="inlineStr"/>
       <c r="Y161" s="6" t="inlineStr"/>
       <c r="Z161" s="6" t="inlineStr"/>
+      <c r="AA161" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21 Construction Owners. Arch-Con Tops Out 330-Unit Artis Montrose Apartment Project  https://www.constructionowners.com/news/arch-con-reaches-topping-out-milestone-on-330-unit-artis-montrose-apartment-project</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="12" t="inlineStr">
@@ -18206,6 +18499,11 @@
       <c r="X162" s="12" t="inlineStr"/>
       <c r="Y162" s="12" t="inlineStr"/>
       <c r="Z162" s="12" t="inlineStr"/>
+      <c r="AA162" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-21 Construction Owners. Arch-Con Tops Out 330-Unit Artis Montrose Apartment Project  https://www.constructionowners.com/news/arch-con-reaches-topping-out-milestone-on-330-unit-artis-montrose-apartment-project</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="6" t="inlineStr">
@@ -18314,6 +18612,11 @@
       <c r="X163" s="6" t="inlineStr"/>
       <c r="Y163" s="6" t="inlineStr"/>
       <c r="Z163" s="6" t="inlineStr"/>
+      <c r="AA163" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21 Construction Owners. Arch-Con Tops Out 330-Unit Artis Montrose Apartment Project  https://www.constructionowners.com/news/arch-con-reaches-topping-out-milestone-on-330-unit-artis-montrose-apartment-project</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="12" t="inlineStr">
@@ -18422,6 +18725,7 @@
       <c r="X164" s="12" t="inlineStr"/>
       <c r="Y164" s="12" t="inlineStr"/>
       <c r="Z164" s="12" t="inlineStr"/>
+      <c r="AA164" s="12" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
@@ -18535,6 +18839,7 @@
       <c r="X165" s="6" t="inlineStr"/>
       <c r="Y165" s="6" t="inlineStr"/>
       <c r="Z165" s="6" t="inlineStr"/>
+      <c r="AA165" s="6" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="12" t="inlineStr">
@@ -18643,6 +18948,7 @@
       <c r="X166" s="12" t="inlineStr"/>
       <c r="Y166" s="12" t="inlineStr"/>
       <c r="Z166" s="12" t="inlineStr"/>
+      <c r="AA166" s="12" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="6" t="inlineStr">
@@ -18760,6 +19066,7 @@
           <t>https://www.tritenre.com/team</t>
         </is>
       </c>
+      <c r="AA167" s="6" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="12" t="inlineStr">
@@ -18877,6 +19184,7 @@
           <t>https://www.tritenre.com/team</t>
         </is>
       </c>
+      <c r="AA168" s="12" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
@@ -18994,6 +19302,7 @@
           <t>https://www.tritenre.com/team</t>
         </is>
       </c>
+      <c r="AA169" s="6" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="12" t="inlineStr">
@@ -19114,6 +19423,7 @@
           <t>https://www.tritenre.com/team</t>
         </is>
       </c>
+      <c r="AA170" s="12" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
@@ -19231,6 +19541,7 @@
           <t>https://www.radomcapital.com/team</t>
         </is>
       </c>
+      <c r="AA171" s="6" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="12" t="inlineStr">
@@ -19348,6 +19659,7 @@
           <t>https://www.radomcapital.com/team</t>
         </is>
       </c>
+      <c r="AA172" s="12" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="6" t="inlineStr">
@@ -19465,6 +19777,7 @@
           <t>https://www.radomcapital.com/team</t>
         </is>
       </c>
+      <c r="AA173" s="6" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="12" t="inlineStr">
@@ -19581,6 +19894,7 @@
           <t>https://www.dealco.net/about/</t>
         </is>
       </c>
+      <c r="AA174" s="12" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="6" t="inlineStr">
@@ -19701,6 +20015,7 @@
           <t>https://cameronmanagement.com/about</t>
         </is>
       </c>
+      <c r="AA175" s="6" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="12" t="inlineStr">
@@ -19821,6 +20136,7 @@
           <t>https://cameronmanagement.com/about</t>
         </is>
       </c>
+      <c r="AA176" s="12" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="6" t="inlineStr">
@@ -19933,6 +20249,7 @@
       </c>
       <c r="Y177" s="6" t="inlineStr"/>
       <c r="Z177" s="6" t="inlineStr"/>
+      <c r="AA177" s="6" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="12" t="inlineStr">
@@ -20046,6 +20363,7 @@
       <c r="X178" s="12" t="inlineStr"/>
       <c r="Y178" s="12" t="inlineStr"/>
       <c r="Z178" s="12" t="inlineStr"/>
+      <c r="AA178" s="12" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="6" t="inlineStr">
@@ -20158,6 +20476,7 @@
       </c>
       <c r="Y179" s="6" t="inlineStr"/>
       <c r="Z179" s="6" t="inlineStr"/>
+      <c r="AA179" s="6" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="12" t="inlineStr">
@@ -20267,6 +20586,7 @@
       <c r="X180" s="12" t="inlineStr"/>
       <c r="Y180" s="12" t="inlineStr"/>
       <c r="Z180" s="12" t="inlineStr"/>
+      <c r="AA180" s="12" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
@@ -20387,6 +20707,7 @@
           <t>https://www.midway.team/our-people</t>
         </is>
       </c>
+      <c r="AA181" s="6" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="12" t="inlineStr">
@@ -20504,6 +20825,7 @@
           <t>https://www.midway.team/our-people</t>
         </is>
       </c>
+      <c r="AA182" s="12" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="6" t="inlineStr">
@@ -20624,6 +20946,7 @@
           <t>https://www.midway.team/our-people</t>
         </is>
       </c>
+      <c r="AA183" s="6" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="12" t="inlineStr">
@@ -20745,6 +21068,7 @@
           <t>https://www.midway.team/our-people</t>
         </is>
       </c>
+      <c r="AA184" s="12" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="6" t="inlineStr">
@@ -20862,6 +21186,7 @@
           <t>https://www.midway.team/our-people</t>
         </is>
       </c>
+      <c r="AA185" s="6" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="12" t="inlineStr">
@@ -20974,6 +21299,7 @@
       </c>
       <c r="Y186" s="12" t="inlineStr"/>
       <c r="Z186" s="12" t="inlineStr"/>
+      <c r="AA186" s="12" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="6" t="inlineStr">
@@ -21087,6 +21413,7 @@
       </c>
       <c r="Y187" s="6" t="inlineStr"/>
       <c r="Z187" s="6" t="inlineStr"/>
+      <c r="AA187" s="6" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="12" t="inlineStr">
@@ -21199,6 +21526,7 @@
       </c>
       <c r="Y188" s="12" t="inlineStr"/>
       <c r="Z188" s="12" t="inlineStr"/>
+      <c r="AA188" s="12" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
@@ -21312,6 +21640,7 @@
       </c>
       <c r="Y189" s="6" t="inlineStr"/>
       <c r="Z189" s="6" t="inlineStr"/>
+      <c r="AA189" s="6" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="12" t="inlineStr">
@@ -21425,6 +21754,7 @@
       </c>
       <c r="Y190" s="12" t="inlineStr"/>
       <c r="Z190" s="12" t="inlineStr"/>
+      <c r="AA190" s="12" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="6" t="inlineStr">
@@ -21538,6 +21868,7 @@
       </c>
       <c r="Y191" s="6" t="inlineStr"/>
       <c r="Z191" s="6" t="inlineStr"/>
+      <c r="AA191" s="6" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="12" t="inlineStr">
@@ -21651,6 +21982,7 @@
       </c>
       <c r="Y192" s="12" t="inlineStr"/>
       <c r="Z192" s="12" t="inlineStr"/>
+      <c r="AA192" s="12" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
@@ -21764,6 +22096,7 @@
       </c>
       <c r="Y193" s="6" t="inlineStr"/>
       <c r="Z193" s="6" t="inlineStr"/>
+      <c r="AA193" s="6" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="12" t="inlineStr">
@@ -21884,6 +22217,7 @@
           <t>https://investor.lgihomes.com/corporate-governance/management</t>
         </is>
       </c>
+      <c r="AA194" s="12" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="6" t="inlineStr">
@@ -22004,6 +22338,7 @@
           <t>https://investor.lgihomes.com/corporate-governance/management</t>
         </is>
       </c>
+      <c r="AA195" s="6" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="12" t="inlineStr">
@@ -22124,6 +22459,7 @@
           <t>https://investor.lgihomes.com/corporate-governance/management</t>
         </is>
       </c>
+      <c r="AA196" s="12" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="6" t="inlineStr">
@@ -22245,6 +22581,7 @@
           <t>https://investor.lgihomes.com/corporate-governance/management</t>
         </is>
       </c>
+      <c r="AA197" s="6" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="12" t="inlineStr">
@@ -22366,6 +22703,7 @@
           <t>https://investor.lgihomes.com/corporate-governance/management</t>
         </is>
       </c>
+      <c r="AA198" s="12" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
@@ -22486,6 +22824,7 @@
           <t>https://investors.mihomes.com/investor-relations/officers-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA199" s="6" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="12" t="inlineStr">
@@ -22606,6 +22945,7 @@
           <t>https://investors.mihomes.com/investor-relations/officers-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA200" s="12" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
@@ -22727,6 +23067,7 @@
           <t>https://investors.mihomes.com/investor-relations/officers-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA201" s="6" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="12" t="inlineStr">
@@ -22848,6 +23189,7 @@
           <t>https://investors.mihomes.com/investor-relations/officers-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA202" s="12" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="6" t="inlineStr">
@@ -22968,6 +23310,7 @@
           <t>https://newsroom.taylormorrison.com/Leadership</t>
         </is>
       </c>
+      <c r="AA203" s="6" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="12" t="inlineStr">
@@ -23081,6 +23424,7 @@
           <t>https://newsroom.taylormorrison.com/Leadership</t>
         </is>
       </c>
+      <c r="AA204" s="12" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="6" t="inlineStr">
@@ -23201,6 +23545,7 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
+      <c r="AA205" s="6" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="12" t="inlineStr">
@@ -23321,6 +23666,7 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
+      <c r="AA206" s="12" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="6" t="inlineStr">
@@ -23441,6 +23787,7 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
+      <c r="AA207" s="6" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="12" t="inlineStr">
@@ -23562,6 +23909,7 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
+      <c r="AA208" s="12" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="6" t="inlineStr">
@@ -23679,6 +24027,7 @@
           <t>https://www.davidweekleyhomes.com/about-us/meet-the-team</t>
         </is>
       </c>
+      <c r="AA209" s="6" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="12" t="inlineStr">
@@ -23799,6 +24148,7 @@
           <t>https://www.davidweekleyhomes.com/about-us/meet-the-team</t>
         </is>
       </c>
+      <c r="AA210" s="12" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="6" t="inlineStr">
@@ -23919,6 +24269,7 @@
           <t>https://www.davidweekleyhomes.com/about-us/meet-the-team</t>
         </is>
       </c>
+      <c r="AA211" s="6" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="12" t="inlineStr">
@@ -24040,6 +24391,7 @@
           <t>https://www.davidweekleyhomes.com/about-us/meet-the-team</t>
         </is>
       </c>
+      <c r="AA212" s="12" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="6" t="inlineStr">
@@ -24157,6 +24509,7 @@
           <t>https://www.davidweekleyhomes.com/about-us/meet-the-team</t>
         </is>
       </c>
+      <c r="AA213" s="6" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="12" t="inlineStr">
@@ -24274,6 +24627,7 @@
           <t>https://www.davidweekleyhomes.com/about-us/meet-the-team</t>
         </is>
       </c>
+      <c r="AA214" s="12" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
@@ -24394,6 +24748,7 @@
           <t>https://www.perryhomes.com/about-perry-homes</t>
         </is>
       </c>
+      <c r="AA215" s="6" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="12" t="inlineStr">
@@ -24514,6 +24869,7 @@
           <t>https://www.perryhomes.com/about-perry-homes</t>
         </is>
       </c>
+      <c r="AA216" s="12" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
@@ -24635,6 +24991,7 @@
           <t>https://www.perryhomes.com/about-perry-homes</t>
         </is>
       </c>
+      <c r="AA217" s="6" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="12" t="inlineStr">
@@ -24756,6 +25113,7 @@
           <t>https://www.perryhomes.com/about-perry-homes</t>
         </is>
       </c>
+      <c r="AA218" s="12" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
@@ -24876,6 +25234,7 @@
           <t>https://www.drbgroup.com/about</t>
         </is>
       </c>
+      <c r="AA219" s="6" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="12" t="inlineStr">
@@ -25001,6 +25360,7 @@
           <t>https://www.drbgroup.com/about</t>
         </is>
       </c>
+      <c r="AA220" s="12" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
@@ -25106,6 +25466,7 @@
           <t>https://www.signorellicompany.com/our-leadership</t>
         </is>
       </c>
+      <c r="AA221" s="6" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="12" t="inlineStr">
@@ -25214,6 +25575,7 @@
           <t>https://www.signorellicompany.com/our-leadership</t>
         </is>
       </c>
+      <c r="AA222" s="12" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
@@ -25322,6 +25684,7 @@
           <t>https://www.signorellicompany.com/our-leadership</t>
         </is>
       </c>
+      <c r="AA223" s="6" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="12" t="inlineStr">
@@ -25430,6 +25793,7 @@
           <t>https://www.signorellicompany.com/our-leadership</t>
         </is>
       </c>
+      <c r="AA224" s="12" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
@@ -25538,6 +25902,7 @@
           <t>https://investor.howardhughes.com/governance/leadership</t>
         </is>
       </c>
+      <c r="AA225" s="6" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="12" t="inlineStr">
@@ -25646,6 +26011,7 @@
           <t>https://investor.howardhughes.com/governance/leadership</t>
         </is>
       </c>
+      <c r="AA226" s="12" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="6" t="inlineStr">
@@ -25754,6 +26120,7 @@
           <t>https://investor.howardhughes.com/governance/leadership</t>
         </is>
       </c>
+      <c r="AA227" s="6" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="12" t="inlineStr">
@@ -25859,6 +26226,7 @@
           <t>https://investor.howardhughes.com/governance/leadership</t>
         </is>
       </c>
+      <c r="AA228" s="12" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
@@ -25963,6 +26331,7 @@
           <t>https://landtejas.com/about-us/our-leadership/</t>
         </is>
       </c>
+      <c r="AA229" s="6" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="12" t="inlineStr">
@@ -26067,6 +26436,7 @@
           <t>https://landtejas.com/about-us/our-leadership/</t>
         </is>
       </c>
+      <c r="AA230" s="12" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="6" t="inlineStr">
@@ -26175,6 +26545,7 @@
           <t>https://caldwellcos.com/our-team</t>
         </is>
       </c>
+      <c r="AA231" s="6" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="12" t="inlineStr">
@@ -26283,6 +26654,7 @@
           <t>https://www.johnsondevelopment.com/our-leaders</t>
         </is>
       </c>
+      <c r="AA232" s="12" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="6" t="inlineStr">
@@ -26387,6 +26759,7 @@
         </is>
       </c>
       <c r="Z233" s="6" t="inlineStr"/>
+      <c r="AA233" s="6" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="12" t="inlineStr">
@@ -26496,6 +26869,7 @@
       <c r="X234" s="12" t="inlineStr"/>
       <c r="Y234" s="12" t="inlineStr"/>
       <c r="Z234" s="12" t="inlineStr"/>
+      <c r="AA234" s="12" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="6" t="inlineStr">
@@ -26616,6 +26990,7 @@
           <t>https://friendswooddevelopment.com/people</t>
         </is>
       </c>
+      <c r="AA235" s="6" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="12" t="inlineStr">
@@ -26724,6 +27099,7 @@
           <t>https://www.newquest.com/about-us/leadership/</t>
         </is>
       </c>
+      <c r="AA236" s="12" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="6" t="inlineStr">
@@ -26832,6 +27208,7 @@
           <t>https://www.newquest.com/about-us/leadership/</t>
         </is>
       </c>
+      <c r="AA237" s="6" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="12" t="inlineStr">
@@ -26940,6 +27317,7 @@
           <t>https://www.newquest.com/about-us/leadership/</t>
         </is>
       </c>
+      <c r="AA238" s="12" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="6" t="inlineStr">
@@ -27048,6 +27426,7 @@
           <t>https://www.newquest.com/about-us/leadership/</t>
         </is>
       </c>
+      <c r="AA239" s="6" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="12" t="inlineStr">
@@ -27156,6 +27535,7 @@
           <t>https://www.frpltd.com/about-fidelis/mission-values</t>
         </is>
       </c>
+      <c r="AA240" s="12" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="6" t="inlineStr">
@@ -27264,6 +27644,7 @@
           <t>https://www.frpltd.com/about-fidelis/mission-values</t>
         </is>
       </c>
+      <c r="AA241" s="6" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="12" t="inlineStr">
@@ -27373,6 +27754,7 @@
           <t>https://www.frpltd.com/about-fidelis/mission-values</t>
         </is>
       </c>
+      <c r="AA242" s="12" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
@@ -27477,6 +27859,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA243" s="6" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="12" t="inlineStr">
@@ -27581,6 +27964,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA244" s="12" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
@@ -27685,6 +28069,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA245" s="6" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="12" t="inlineStr">
@@ -27789,6 +28174,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA246" s="12" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
@@ -27894,6 +28280,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA247" s="6" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="12" t="inlineStr">
@@ -27999,6 +28386,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA248" s="12" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
@@ -28104,6 +28492,7 @@
           <t>https://www.hanoverco.com/leadership</t>
         </is>
       </c>
+      <c r="AA249" s="6" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="12" t="inlineStr">
@@ -28212,6 +28601,7 @@
           <t>https://www.read-king.com/team</t>
         </is>
       </c>
+      <c r="AA250" s="12" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="6" t="inlineStr">
@@ -28320,6 +28710,7 @@
           <t>https://www.read-king.com/team</t>
         </is>
       </c>
+      <c r="AA251" s="6" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="12" t="inlineStr">
@@ -28428,6 +28819,7 @@
           <t>https://www.read-king.com/team</t>
         </is>
       </c>
+      <c r="AA252" s="12" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="6" t="inlineStr">
@@ -28533,6 +28925,7 @@
           <t>https://www.read-king.com/team</t>
         </is>
       </c>
+      <c r="AA253" s="6" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="12" t="inlineStr">
@@ -28641,6 +29034,7 @@
           <t>https://investors.camdenliving.com/investors/governance/board-of-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA254" s="12" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="6" t="inlineStr">
@@ -28749,6 +29143,7 @@
           <t>https://investors.camdenliving.com/investors/governance/board-of-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA255" s="6" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="12" t="inlineStr">
@@ -28858,6 +29253,7 @@
           <t>https://investors.camdenliving.com/investors/governance/board-of-directors/default.aspx</t>
         </is>
       </c>
+      <c r="AA256" s="12" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="6" t="inlineStr">
@@ -28966,6 +29362,7 @@
           <t>https://www.greystar.com/business/about-greystar/our-leadership</t>
         </is>
       </c>
+      <c r="AA257" s="6" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="12" t="inlineStr">
@@ -29074,6 +29471,7 @@
           <t>https://www.greystar.com/business/about-greystar/our-leadership</t>
         </is>
       </c>
+      <c r="AA258" s="12" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="6" t="inlineStr">
@@ -29182,6 +29580,7 @@
           <t>https://www.dinersteincos.com/about-us</t>
         </is>
       </c>
+      <c r="AA259" s="6" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="12" t="inlineStr">
@@ -29287,6 +29686,7 @@
           <t>https://www.dinersteincos.com/about-us</t>
         </is>
       </c>
+      <c r="AA260" s="12" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="6" t="inlineStr">
@@ -29395,6 +29795,7 @@
           <t>https://www.dinersteincos.com/about-us</t>
         </is>
       </c>
+      <c r="AA261" s="6" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="12" t="inlineStr">
@@ -29503,6 +29904,7 @@
           <t>https://www.dinersteincos.com/about-us</t>
         </is>
       </c>
+      <c r="AA262" s="12" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
@@ -29603,6 +30005,7 @@
           <t>https://bakerkatz.com/about-us/</t>
         </is>
       </c>
+      <c r="AA263" s="6" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="12" t="inlineStr">
@@ -29703,6 +30106,7 @@
           <t>https://bakerkatz.com/about-us/</t>
         </is>
       </c>
+      <c r="AA264" s="12" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="6" t="inlineStr">
@@ -29807,6 +30211,7 @@
           <t>https://bakerkatz.com/about-us/</t>
         </is>
       </c>
+      <c r="AA265" s="6" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="12" t="inlineStr">
@@ -29907,6 +30312,7 @@
           <t>https://www.wulfe.com/people</t>
         </is>
       </c>
+      <c r="AA266" s="12" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="6" t="inlineStr">
@@ -30011,16 +30417,17 @@
           <t>https://www.wulfe.com/people</t>
         </is>
       </c>
+      <c r="AA267" s="6" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 39, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 40, 2026-09-11.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:Z267"/>
+  <autoFilter ref="A6:AA267"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build 42: an absence is a blank, not a sentence
The page no longer narrates what it does not have. "none published" is gone from
the decision-maker cell and the print roster, the two limits blocks that
explained empty fields and counted the firms publishing nobody are deleted, and
the press block no longer names the firms that returned nothing. Ten limits
blocks became eight. The .yn.none rule came out of the stylesheet.

Absences that explain a mark the reader can see stayed: the band rule that makes
an unpublished figure a Partly, and the block behind the decider caveat chip.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -565,7 +565,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 41 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 42 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -28877,7 +28877,7 @@
     <row r="266">
       <c r="A266" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 41, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 42, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 43: the subtraction pass
Twenty-eight sentences off the deck. The score narrating itself (the zero
records an absent search result), a sentence for a cell that was already blank,
and screen lines restating a count chip the reader can see. Three limits blocks
lost a closing clause of the same kind.

Absences that are findings stayed: no third party in the method decision, no
Houston site named, no outside architect credited, no US factory. Those carry a
proper noun or contradict an assumption.

Also out: two lines that told the reader what to conclude, and Midway's screen
ending on an open item that the record had already resolved.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -565,7 +565,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 42 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 43 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="T55" s="9" t="inlineStr">
         <is>
-          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters. No wall-system statement on record.</t>
+          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters.</t>
         </is>
       </c>
       <c r="U55" s="6" t="inlineStr"/>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="T56" s="15" t="inlineStr">
         <is>
-          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters. No wall-system statement on record.</t>
+          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters.</t>
         </is>
       </c>
       <c r="U56" s="12" t="inlineStr"/>
@@ -6496,7 +6496,7 @@
       </c>
       <c r="T57" s="9" t="inlineStr">
         <is>
-          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters. No wall-system statement on record.</t>
+          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters.</t>
         </is>
       </c>
       <c r="U57" s="6" t="inlineStr"/>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="T58" s="15" t="inlineStr">
         <is>
-          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters. No wall-system statement on record.</t>
+          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters.</t>
         </is>
       </c>
       <c r="U58" s="12" t="inlineStr">
@@ -6730,7 +6730,7 @@
       </c>
       <c r="T59" s="9" t="inlineStr">
         <is>
-          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters. No wall-system statement on record.</t>
+          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters.</t>
         </is>
       </c>
       <c r="U59" s="6" t="inlineStr"/>
@@ -6843,7 +6843,7 @@
       </c>
       <c r="T60" s="15" t="inlineStr">
         <is>
-          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters. No wall-system statement on record.</t>
+          <t>1,000 homes at Trinity Landing and a sub-110-day cycle held four quarters.</t>
         </is>
       </c>
       <c r="U60" s="12" t="inlineStr"/>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="T62" s="15" t="inlineStr">
         <is>
-          <t>10,800 rental homes across 115 communities, built and held. No construction-method statement anywhere.</t>
+          <t>10,800 rental homes across 115 communities, built and held.</t>
         </is>
       </c>
       <c r="U62" s="12" t="inlineStr"/>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="T63" s="9" t="inlineStr">
         <is>
-          <t>10,800 rental homes across 115 communities, built and held. No construction-method statement anywhere.</t>
+          <t>10,800 rental homes across 115 communities, built and held.</t>
         </is>
       </c>
       <c r="U63" s="6" t="inlineStr"/>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="T64" s="15" t="inlineStr">
         <is>
-          <t>10,800 rental homes across 115 communities, built and held. No construction-method statement anywhere.</t>
+          <t>10,800 rental homes across 115 communities, built and held.</t>
         </is>
       </c>
       <c r="U64" s="12" t="inlineStr"/>
@@ -7411,7 +7411,7 @@
       </c>
       <c r="T65" s="9" t="inlineStr">
         <is>
-          <t>10,800 rental homes across 115 communities, built and held. No construction-method statement anywhere.</t>
+          <t>10,800 rental homes across 115 communities, built and held.</t>
         </is>
       </c>
       <c r="U65" s="6" t="inlineStr"/>
@@ -7527,7 +7527,7 @@
       </c>
       <c r="T66" s="15" t="inlineStr">
         <is>
-          <t>20,000 homes since 2004. Daiwa House owns a stake. No published method evidence.</t>
+          <t>20,000 homes since 2004. Daiwa House owns a stake.</t>
         </is>
       </c>
       <c r="U66" s="12" t="inlineStr"/>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="T67" s="9" t="inlineStr">
         <is>
-          <t>20,000 homes since 2004. Daiwa House owns a stake. No published method evidence.</t>
+          <t>20,000 homes since 2004. Daiwa House owns a stake.</t>
         </is>
       </c>
       <c r="U67" s="6" t="inlineStr"/>
@@ -7757,7 +7757,7 @@
       </c>
       <c r="T68" s="15" t="inlineStr">
         <is>
-          <t>20,000 homes since 2004. Daiwa House owns a stake. No published method evidence.</t>
+          <t>20,000 homes since 2004. Daiwa House owns a stake.</t>
         </is>
       </c>
       <c r="U68" s="12" t="inlineStr"/>
@@ -9785,7 +9785,7 @@
       </c>
       <c r="T87" s="9" t="inlineStr">
         <is>
-          <t>Seven plans, ten communities, founded 2020. No closings figure to size it against.</t>
+          <t>Seven plans, ten communities, founded 2020.</t>
         </is>
       </c>
       <c r="U87" s="6" t="inlineStr"/>
@@ -9885,7 +9885,7 @@
       </c>
       <c r="T88" s="15" t="inlineStr">
         <is>
-          <t>Seven plans, ten communities, founded 2020. No closings figure to size it against.</t>
+          <t>Seven plans, ten communities, founded 2020.</t>
         </is>
       </c>
       <c r="U88" s="12" t="inlineStr"/>
@@ -9986,7 +9986,7 @@
       </c>
       <c r="T89" s="9" t="inlineStr">
         <is>
-          <t>Seven plans, ten communities, founded 2020. No closings figure to size it against.</t>
+          <t>Seven plans, ten communities, founded 2020.</t>
         </is>
       </c>
       <c r="U89" s="6" t="inlineStr">
@@ -10327,7 +10327,7 @@
       </c>
       <c r="T92" s="15" t="inlineStr">
         <is>
-          <t>A national platform with a Houston division president who is a licensed engineer. One community identified so far.</t>
+          <t>A national platform with a Houston division president who is a licensed engineer, building in Sunterra.</t>
         </is>
       </c>
       <c r="U92" s="12" t="inlineStr"/>
@@ -10436,7 +10436,7 @@
       </c>
       <c r="T93" s="9" t="inlineStr">
         <is>
-          <t>A national platform with a Houston division president who is a licensed engineer. One community identified so far.</t>
+          <t>A national platform with a Houston division president who is a licensed engineer, building in Sunterra.</t>
         </is>
       </c>
       <c r="U93" s="6" t="inlineStr"/>
@@ -10545,7 +10545,7 @@
       </c>
       <c r="T94" s="15" t="inlineStr">
         <is>
-          <t>Close to 100 communities inside Dream Finders, which bought parent MHI in 2021. Two Houston division presidents are named.</t>
+          <t>Close to 100 communities inside Dream Finders, which bought parent MHI in 2021.</t>
         </is>
       </c>
       <c r="U94" s="12" t="inlineStr"/>
@@ -10654,7 +10654,7 @@
       </c>
       <c r="T95" s="9" t="inlineStr">
         <is>
-          <t>Close to 100 communities inside Dream Finders, which bought parent MHI in 2021. Two Houston division presidents are named.</t>
+          <t>Close to 100 communities inside Dream Finders, which bought parent MHI in 2021.</t>
         </is>
       </c>
       <c r="U95" s="6" t="inlineStr"/>
@@ -10762,7 +10762,7 @@
       </c>
       <c r="T96" s="15" t="inlineStr">
         <is>
-          <t>483 closings in 2025 across more than twenty communities and more than 150 plans. A president is named; no construction or purchasing lead is published.</t>
+          <t>483 closings in 2025 across more than twenty communities and more than 150 plans.</t>
         </is>
       </c>
       <c r="U96" s="12" t="inlineStr"/>
@@ -11402,7 +11402,7 @@
       </c>
       <c r="T102" s="15" t="inlineStr">
         <is>
-          <t>Two Katy duplex projects a mile apart, 366 units. No capital figure and no method evidence.</t>
+          <t>Two Katy duplex projects a mile apart, 366 units.</t>
         </is>
       </c>
       <c r="U102" s="12" t="inlineStr"/>
@@ -11518,7 +11518,7 @@
       </c>
       <c r="T103" s="9" t="inlineStr">
         <is>
-          <t>Two Katy duplex projects a mile apart, 366 units. No capital figure and no method evidence.</t>
+          <t>Two Katy duplex projects a mile apart, 366 units.</t>
         </is>
       </c>
       <c r="U103" s="6" t="inlineStr">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="T104" s="15" t="inlineStr">
         <is>
-          <t>Two Katy duplex projects a mile apart, 366 units. No capital figure and no method evidence.</t>
+          <t>Two Katy duplex projects a mile apart, 366 units.</t>
         </is>
       </c>
       <c r="U104" s="12" t="inlineStr"/>
@@ -19536,7 +19536,7 @@
       </c>
       <c r="T178" s="15" t="inlineStr">
         <is>
-          <t>East River is 60 blocks on one site. No capital figure disclosed and the Parkway relationship is unresolved.</t>
+          <t>East River is 60 blocks on one site, and Midway kept sole development control after selling out of the Parkway joint venture in December 2024.</t>
         </is>
       </c>
       <c r="U178" s="12" t="inlineStr"/>
@@ -19653,7 +19653,7 @@
       </c>
       <c r="T179" s="9" t="inlineStr">
         <is>
-          <t>East River is 60 blocks on one site. No capital figure disclosed and the Parkway relationship is unresolved.</t>
+          <t>East River is 60 blocks on one site, and Midway kept sole development control after selling out of the Parkway joint venture in December 2024.</t>
         </is>
       </c>
       <c r="U179" s="6" t="inlineStr"/>
@@ -19765,7 +19765,7 @@
       </c>
       <c r="T180" s="15" t="inlineStr">
         <is>
-          <t>East River is 60 blocks on one site. No capital figure disclosed and the Parkway relationship is unresolved.</t>
+          <t>East River is 60 blocks on one site, and Midway kept sole development control after selling out of the Parkway joint venture in December 2024.</t>
         </is>
       </c>
       <c r="U180" s="12" t="inlineStr"/>
@@ -19882,7 +19882,7 @@
       </c>
       <c r="T181" s="9" t="inlineStr">
         <is>
-          <t>East River is 60 blocks on one site. No capital figure disclosed and the Parkway relationship is unresolved.</t>
+          <t>East River is 60 blocks on one site, and Midway kept sole development control after selling out of the Parkway joint venture in December 2024.</t>
         </is>
       </c>
       <c r="U181" s="6" t="inlineStr">
@@ -19999,7 +19999,7 @@
       </c>
       <c r="T182" s="15" t="inlineStr">
         <is>
-          <t>East River is 60 blocks on one site. No capital figure disclosed and the Parkway relationship is unresolved.</t>
+          <t>East River is 60 blocks on one site, and Midway kept sole development control after selling out of the Parkway joint venture in December 2024.</t>
         </is>
       </c>
       <c r="U182" s="12" t="inlineStr"/>
@@ -22258,7 +22258,7 @@
       </c>
       <c r="T202" s="15" t="inlineStr">
         <is>
-          <t>14 named Houston communities and a Texas regional president. No firm-specific method evidence found.</t>
+          <t>14 named Houston communities and a Texas regional president.</t>
         </is>
       </c>
       <c r="U202" s="12" t="inlineStr"/>
@@ -22374,7 +22374,7 @@
       </c>
       <c r="T203" s="9" t="inlineStr">
         <is>
-          <t>14 named Houston communities and a Texas regional president. No firm-specific method evidence found.</t>
+          <t>14 named Houston communities and a Texas regional president.</t>
         </is>
       </c>
       <c r="U203" s="6" t="inlineStr"/>
@@ -22490,7 +22490,7 @@
       </c>
       <c r="T204" s="15" t="inlineStr">
         <is>
-          <t>14 named Houston communities and a Texas regional president. No firm-specific method evidence found.</t>
+          <t>14 named Houston communities and a Texas regional president.</t>
         </is>
       </c>
       <c r="U204" s="12" t="inlineStr"/>
@@ -22607,7 +22607,7 @@
       </c>
       <c r="T205" s="9" t="inlineStr">
         <is>
-          <t>14 named Houston communities and a Texas regional president. No firm-specific method evidence found.</t>
+          <t>14 named Houston communities and a Texas regional president.</t>
         </is>
       </c>
       <c r="U205" s="6" t="inlineStr">
@@ -25136,7 +25136,7 @@
       </c>
       <c r="T228" s="15" t="inlineStr">
         <is>
-          <t>Sells lots. Towne Lake and The Highlands carry 4,000 homes across 12 builders. No published method evidence.</t>
+          <t>Sells lots. Towne Lake and The Highlands carry 4,000 homes across 12 builders.</t>
         </is>
       </c>
       <c r="U228" s="12" t="inlineStr"/>
@@ -28877,7 +28877,7 @@
     <row r="266">
       <c r="A266" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 42, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 43, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 45: the map, drawn properly
The outlines were simplified per county, so a shared border came back as two
lines up to 600m apart, which is nearly two pixels at this scale. That is why
every seam read doubled. Outlines are now pulled at about 130m and snapped to
three decimals, under a pixel, so a shared border lands on one line.

Fills carry no stroke; one grey hairline layer draws every boundary above them,
interior and exterior at the same weight. Labels sit at each county's pole of
inaccessibility rather than its centroid. The ramp starts at #EDEDED so the
quietest county still reads. The key is one strip labelled at its ends, and no
longer runs off the edge: .axt sets text-anchor middle in CSS and was overriding
the attribute, so .axs and .axe now exist. Below 700px the map keeps a working
size and scrolls in its own wrapper.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -582,7 +582,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 44 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 45 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -28894,7 +28894,7 @@
     <row r="266">
       <c r="A266" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 44, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 45, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 49: the background, the grid, and a fact printed three times
.bg carries an opaque paper background at z-index:-1 and follows #atmos in the
DOM, so it has painted over the atmosphere canvas since the deck was built. A
hard red rectangle drawn onto the canvas never reached the screen. .bg moves to
z-index:-2. The renderer also still read the Americas deck's tokens and fell
back to a gold not in this palette; it reads --ink now, and the accent stays out
of the ambient layer.

The grid's axes ran outward from the bottom left, so the first cell a reader
lands on held one firm. Columns reversed: top left is now Repetition Yes and
Printer fit Yes. Chips inside each cell order by published annual closings,
largest first, and carry the figure.

An evidence line that only restates the title is dropped at build time. 208
lines became 198.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -582,7 +582,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 48 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 49 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -986,11 +986,7 @@
         </is>
       </c>
       <c r="U8" s="12" t="inlineStr"/>
-      <c r="V8" s="15" t="inlineStr">
-        <is>
-          <t>Co-founder.</t>
-        </is>
-      </c>
+      <c r="V8" s="15" t="inlineStr"/>
       <c r="W8" s="12" t="inlineStr">
         <is>
           <t>https://colekleinbuilders.com/about/</t>
@@ -3053,11 +3049,7 @@
         </is>
       </c>
       <c r="U26" s="12" t="inlineStr"/>
-      <c r="V26" s="15" t="inlineStr">
-        <is>
-          <t>Division President, First America Homes. Houston, Texas.</t>
-        </is>
-      </c>
+      <c r="V26" s="15" t="inlineStr"/>
       <c r="W26" s="12" t="inlineStr"/>
       <c r="X26" s="12" t="inlineStr">
         <is>
@@ -3405,7 +3397,7 @@
       </c>
       <c r="V29" s="9" t="inlineStr">
         <is>
-          <t>Indexed title reads Bruce Hendren, Stylecraft. The firm's team page lists him as Vice President of Pre-Construction. Team page lists Bruce Hendren, Vice President of Pre-Construction.</t>
+          <t>Indexed title reads Bruce Hendren, Stylecraft. The firm's team page lists him as Vice President of Pre-Construction.</t>
         </is>
       </c>
       <c r="W29" s="6" t="inlineStr">
@@ -4608,11 +4600,7 @@
         </is>
       </c>
       <c r="U40" s="12" t="inlineStr"/>
-      <c r="V40" s="15" t="inlineStr">
-        <is>
-          <t>Executive Vice President and Chief Operating Officer.</t>
-        </is>
-      </c>
+      <c r="V40" s="15" t="inlineStr"/>
       <c r="W40" s="12" t="inlineStr">
         <is>
           <t>https://suebausa.com/about-us/</t>
@@ -9368,11 +9356,7 @@
         </is>
       </c>
       <c r="U83" s="6" t="inlineStr"/>
-      <c r="V83" s="9" t="inlineStr">
-        <is>
-          <t>Team page: Co-President.</t>
-        </is>
-      </c>
+      <c r="V83" s="9" t="inlineStr"/>
       <c r="W83" s="6" t="inlineStr">
         <is>
           <t>https://jamestownestatehomes.com/team/katy-hawes/</t>
@@ -9476,11 +9460,7 @@
         </is>
       </c>
       <c r="U84" s="12" t="inlineStr"/>
-      <c r="V84" s="15" t="inlineStr">
-        <is>
-          <t>Team page: Co-President.</t>
-        </is>
-      </c>
+      <c r="V84" s="15" t="inlineStr"/>
       <c r="W84" s="12" t="inlineStr">
         <is>
           <t>https://jamestownestatehomes.com/team/matt-norris/</t>
@@ -10459,7 +10439,7 @@
       <c r="U93" s="6" t="inlineStr"/>
       <c r="V93" s="9" t="inlineStr">
         <is>
-          <t>Indexed title reads Matthew Zaist, President and CEO at Risewell Homes. Confirmed on the firm's team page. Executive team page: President and Chief Executive Officer.</t>
+          <t>Indexed title reads Matthew Zaist, President and CEO at Risewell Homes. Confirmed on the firm's team page.</t>
         </is>
       </c>
       <c r="W93" s="6" t="inlineStr">
@@ -11423,11 +11403,7 @@
         </is>
       </c>
       <c r="U102" s="12" t="inlineStr"/>
-      <c r="V102" s="15" t="inlineStr">
-        <is>
-          <t>Managing Member.</t>
-        </is>
-      </c>
+      <c r="V102" s="15" t="inlineStr"/>
       <c r="W102" s="12" t="inlineStr">
         <is>
           <t>https://rskrealestatepartners.com/our-team/</t>
@@ -11659,11 +11635,7 @@
         </is>
       </c>
       <c r="U104" s="12" t="inlineStr"/>
-      <c r="V104" s="15" t="inlineStr">
-        <is>
-          <t>Vice President of Development.</t>
-        </is>
-      </c>
+      <c r="V104" s="15" t="inlineStr"/>
       <c r="W104" s="12" t="inlineStr">
         <is>
           <t>https://rskrealestatepartners.com/our-team/</t>
@@ -18445,11 +18417,7 @@
         </is>
       </c>
       <c r="U168" s="12" t="inlineStr"/>
-      <c r="V168" s="15" t="inlineStr">
-        <is>
-          <t>Managing Principal at Radom Capital.</t>
-        </is>
-      </c>
+      <c r="V168" s="15" t="inlineStr"/>
       <c r="W168" s="12" t="inlineStr"/>
       <c r="X168" s="12" t="inlineStr">
         <is>
@@ -19786,11 +19754,7 @@
         </is>
       </c>
       <c r="U180" s="12" t="inlineStr"/>
-      <c r="V180" s="15" t="inlineStr">
-        <is>
-          <t>Executive Vice President and General Counsel.</t>
-        </is>
-      </c>
+      <c r="V180" s="15" t="inlineStr"/>
       <c r="W180" s="12" t="inlineStr">
         <is>
           <t>https://www.midway.team/our-people</t>
@@ -20020,11 +19984,7 @@
         </is>
       </c>
       <c r="U182" s="12" t="inlineStr"/>
-      <c r="V182" s="15" t="inlineStr">
-        <is>
-          <t>Executive Vice President, Midway. Houston, Texas.</t>
-        </is>
-      </c>
+      <c r="V182" s="15" t="inlineStr"/>
       <c r="W182" s="12" t="inlineStr"/>
       <c r="X182" s="12" t="inlineStr">
         <is>
@@ -20132,11 +20092,7 @@
         </is>
       </c>
       <c r="U183" s="6" t="inlineStr"/>
-      <c r="V183" s="9" t="inlineStr">
-        <is>
-          <t>Team page: Founder and Managing Principal.</t>
-        </is>
-      </c>
+      <c r="V183" s="9" t="inlineStr"/>
       <c r="W183" s="6" t="inlineStr">
         <is>
           <t>https://www.pagewood.com/team</t>
@@ -20243,7 +20199,7 @@
       <c r="U184" s="12" t="inlineStr"/>
       <c r="V184" s="15" t="inlineStr">
         <is>
-          <t>Indexed title reads Mathew Volz, Managing Principal at Pagewood. The firm's team page spells the name Mat. Team page: Managing Principal.</t>
+          <t>Indexed title reads Mathew Volz, Managing Principal at Pagewood. The firm's team page spells the name Mat.</t>
         </is>
       </c>
       <c r="W184" s="12" t="inlineStr">
@@ -20349,11 +20305,7 @@
         </is>
       </c>
       <c r="U185" s="6" t="inlineStr"/>
-      <c r="V185" s="9" t="inlineStr">
-        <is>
-          <t>Team page: Senior Construction Manager.</t>
-        </is>
-      </c>
+      <c r="V185" s="9" t="inlineStr"/>
       <c r="W185" s="6" t="inlineStr">
         <is>
           <t>https://www.pagewood.com/team</t>
@@ -20458,11 +20410,7 @@
         </is>
       </c>
       <c r="U186" s="12" t="inlineStr"/>
-      <c r="V186" s="15" t="inlineStr">
-        <is>
-          <t>Linked from conceptneighborhood.com/team, which lists him as Managing Partner, Projects and Finance. Team page: Managing Partner, Projects and Finance.</t>
-        </is>
-      </c>
+      <c r="V186" s="15" t="inlineStr"/>
       <c r="W186" s="12" t="inlineStr">
         <is>
           <t>https://www.conceptneighborhood.com/team</t>
@@ -20567,11 +20515,7 @@
         </is>
       </c>
       <c r="U187" s="6" t="inlineStr"/>
-      <c r="V187" s="9" t="inlineStr">
-        <is>
-          <t>Linked from conceptneighborhood.com/team, which lists him as Managing Partner, Brokerage and Placemaking. Team page: Managing Partner, Brokerage and Placemaking.</t>
-        </is>
-      </c>
+      <c r="V187" s="9" t="inlineStr"/>
       <c r="W187" s="6" t="inlineStr">
         <is>
           <t>https://www.conceptneighborhood.com/team</t>
@@ -20676,11 +20620,7 @@
         </is>
       </c>
       <c r="U188" s="12" t="inlineStr"/>
-      <c r="V188" s="15" t="inlineStr">
-        <is>
-          <t>Linked from conceptneighborhood.com/team, which lists him as Partner, Design and Placemaking. Team page: Partner, Design and Placemaking.</t>
-        </is>
-      </c>
+      <c r="V188" s="15" t="inlineStr"/>
       <c r="W188" s="12" t="inlineStr">
         <is>
           <t>https://www.conceptneighborhood.com/team</t>
@@ -20785,11 +20725,7 @@
         </is>
       </c>
       <c r="U189" s="6" t="inlineStr"/>
-      <c r="V189" s="9" t="inlineStr">
-        <is>
-          <t>Linked from conceptneighborhood.com/team, which lists him as Managing Partner, Projects and Legal. Team page: Managing Partner, Projects and Legal.</t>
-        </is>
-      </c>
+      <c r="V189" s="9" t="inlineStr"/>
       <c r="W189" s="6" t="inlineStr">
         <is>
           <t>https://www.conceptneighborhood.com/team</t>
@@ -21938,11 +21874,7 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="V199" s="9" t="inlineStr">
-        <is>
-          <t>Vice President of Purchasing, M/I Homes - Houston. Houston, Texas.</t>
-        </is>
-      </c>
+      <c r="V199" s="9" t="inlineStr"/>
       <c r="W199" s="6" t="inlineStr"/>
       <c r="X199" s="6" t="inlineStr">
         <is>
@@ -22279,11 +22211,7 @@
         </is>
       </c>
       <c r="U202" s="12" t="inlineStr"/>
-      <c r="V202" s="15" t="inlineStr">
-        <is>
-          <t>President and Chief Executive Officer.</t>
-        </is>
-      </c>
+      <c r="V202" s="15" t="inlineStr"/>
       <c r="W202" s="12" t="inlineStr">
         <is>
           <t>https://www.ashtonwoods.com/corporate-info</t>
@@ -22511,11 +22439,7 @@
         </is>
       </c>
       <c r="U204" s="12" t="inlineStr"/>
-      <c r="V204" s="15" t="inlineStr">
-        <is>
-          <t>Chief Operating Officer.</t>
-        </is>
-      </c>
+      <c r="V204" s="15" t="inlineStr"/>
       <c r="W204" s="12" t="inlineStr">
         <is>
           <t>https://www.ashtonwoods.com/corporate-info</t>
@@ -23548,11 +23472,7 @@
         </is>
       </c>
       <c r="U213" s="6" t="inlineStr"/>
-      <c r="V213" s="9" t="inlineStr">
-        <is>
-          <t>Chief Executive Officer on Perry's own page.</t>
-        </is>
-      </c>
+      <c r="V213" s="9" t="inlineStr"/>
       <c r="W213" s="6" t="inlineStr">
         <is>
           <t>https://www.perryhomes.com/about-perry-homes</t>
@@ -25174,11 +25094,7 @@
         </is>
       </c>
       <c r="U227" s="6" t="inlineStr"/>
-      <c r="V227" s="9" t="inlineStr">
-        <is>
-          <t>Co-President.</t>
-        </is>
-      </c>
+      <c r="V227" s="9" t="inlineStr"/>
       <c r="W227" s="6" t="inlineStr">
         <is>
           <t>https://landtejas.com/about-us/our-leadership/</t>
@@ -25290,11 +25206,7 @@
         </is>
       </c>
       <c r="U228" s="12" t="inlineStr"/>
-      <c r="V228" s="15" t="inlineStr">
-        <is>
-          <t>Co-President.</t>
-        </is>
-      </c>
+      <c r="V228" s="15" t="inlineStr"/>
       <c r="W228" s="12" t="inlineStr">
         <is>
           <t>https://landtejas.com/about-us/our-leadership/</t>
@@ -25406,11 +25318,7 @@
         </is>
       </c>
       <c r="U229" s="6" t="inlineStr"/>
-      <c r="V229" s="9" t="inlineStr">
-        <is>
-          <t>Chief Executive Officer.</t>
-        </is>
-      </c>
+      <c r="V229" s="9" t="inlineStr"/>
       <c r="W229" s="6" t="inlineStr">
         <is>
           <t>https://caldwellcos.com/our-team</t>
@@ -25522,11 +25430,7 @@
         </is>
       </c>
       <c r="U230" s="12" t="inlineStr"/>
-      <c r="V230" s="15" t="inlineStr">
-        <is>
-          <t>President and Chief Executive Officer.</t>
-        </is>
-      </c>
+      <c r="V230" s="15" t="inlineStr"/>
       <c r="W230" s="12" t="inlineStr">
         <is>
           <t>https://www.johnsondevelopment.com/our-leaders</t>
@@ -25855,11 +25759,7 @@
         </is>
       </c>
       <c r="U233" s="6" t="inlineStr"/>
-      <c r="V233" s="9" t="inlineStr">
-        <is>
-          <t>President.</t>
-        </is>
-      </c>
+      <c r="V233" s="9" t="inlineStr"/>
       <c r="W233" s="6" t="inlineStr">
         <is>
           <t>https://friendswooddevelopment.com/people</t>
@@ -25959,11 +25859,7 @@
         </is>
       </c>
       <c r="U234" s="12" t="inlineStr"/>
-      <c r="V234" s="15" t="inlineStr">
-        <is>
-          <t>Co-Founder and Managing Partner.</t>
-        </is>
-      </c>
+      <c r="V234" s="15" t="inlineStr"/>
       <c r="W234" s="12" t="inlineStr">
         <is>
           <t>https://www.newquest.com/about-us/leadership/</t>
@@ -26063,11 +25959,7 @@
         </is>
       </c>
       <c r="U235" s="6" t="inlineStr"/>
-      <c r="V235" s="9" t="inlineStr">
-        <is>
-          <t>Co-Founder and Managing Partner.</t>
-        </is>
-      </c>
+      <c r="V235" s="9" t="inlineStr"/>
       <c r="W235" s="6" t="inlineStr">
         <is>
           <t>https://www.newquest.com/about-us/leadership/</t>
@@ -26167,11 +26059,7 @@
         </is>
       </c>
       <c r="U236" s="12" t="inlineStr"/>
-      <c r="V236" s="15" t="inlineStr">
-        <is>
-          <t>President and Chief Development Officer.</t>
-        </is>
-      </c>
+      <c r="V236" s="15" t="inlineStr"/>
       <c r="W236" s="12" t="inlineStr">
         <is>
           <t>https://www.newquest.com/about-us/leadership/</t>
@@ -26271,11 +26159,7 @@
         </is>
       </c>
       <c r="U237" s="6" t="inlineStr"/>
-      <c r="V237" s="9" t="inlineStr">
-        <is>
-          <t>Chief Operating Officer and Head of Capital Markets.</t>
-        </is>
-      </c>
+      <c r="V237" s="9" t="inlineStr"/>
       <c r="W237" s="6" t="inlineStr">
         <is>
           <t>https://www.newquest.com/about-us/leadership/</t>
@@ -27391,11 +27275,7 @@
         </is>
       </c>
       <c r="U248" s="12" t="inlineStr"/>
-      <c r="V248" s="15" t="inlineStr">
-        <is>
-          <t>Principal.</t>
-        </is>
-      </c>
+      <c r="V248" s="15" t="inlineStr"/>
       <c r="W248" s="12" t="inlineStr">
         <is>
           <t>https://www.read-king.com/team</t>
@@ -27495,11 +27375,7 @@
         </is>
       </c>
       <c r="U249" s="6" t="inlineStr"/>
-      <c r="V249" s="9" t="inlineStr">
-        <is>
-          <t>Principal.</t>
-        </is>
-      </c>
+      <c r="V249" s="9" t="inlineStr"/>
       <c r="W249" s="6" t="inlineStr">
         <is>
           <t>https://www.read-king.com/team</t>
@@ -27599,11 +27475,7 @@
         </is>
       </c>
       <c r="U250" s="12" t="inlineStr"/>
-      <c r="V250" s="15" t="inlineStr">
-        <is>
-          <t>Chief Financial Officer.</t>
-        </is>
-      </c>
+      <c r="V250" s="15" t="inlineStr"/>
       <c r="W250" s="12" t="inlineStr">
         <is>
           <t>https://www.read-king.com/team</t>
@@ -28530,11 +28402,7 @@
         </is>
       </c>
       <c r="U259" s="6" t="inlineStr"/>
-      <c r="V259" s="9" t="inlineStr">
-        <is>
-          <t>Managing Partner of Development and Design.</t>
-        </is>
-      </c>
+      <c r="V259" s="9" t="inlineStr"/>
       <c r="W259" s="6" t="inlineStr">
         <is>
           <t>https://www.dinersteincos.com/about-us</t>
@@ -28634,11 +28502,7 @@
         </is>
       </c>
       <c r="U260" s="12" t="inlineStr"/>
-      <c r="V260" s="15" t="inlineStr">
-        <is>
-          <t>President and Partner.</t>
-        </is>
-      </c>
+      <c r="V260" s="15" t="inlineStr"/>
       <c r="W260" s="12" t="inlineStr">
         <is>
           <t>https://www.dinersteincos.com/about-us</t>
@@ -29142,11 +29006,7 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="V265" s="9" t="inlineStr">
-        <is>
-          <t>Director of Construction.</t>
-        </is>
-      </c>
+      <c r="V265" s="9" t="inlineStr"/>
       <c r="W265" s="6" t="inlineStr">
         <is>
           <t>https://www.wulfe.com/people</t>
@@ -29167,7 +29027,7 @@
     <row r="267">
       <c r="A267" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 48, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 49, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 57: the number gets its own row, and the section labels grow
Who to call said Who to call and the first thing under it was a phone number,
which is not a who. The people keep that heading. The numbers, their labels,
their source link, the directory and the stated absences move to a row of their
own directly below it, called Phone numbers, which is true in all three states.

The main line now sits on its own line at 22px with its label and source link
on a second line beneath it. They ran together before.

Section labels in the left column go from 10px/600 to 12px/700 and up one step
in contrast.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/ICON_Greater_Houston_Rolodex.xlsx
+++ b/docs/ICON_Greater_Houston_Rolodex.xlsx
@@ -585,7 +585,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from houston-data.json · build 56 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
+          <t>Generated from houston-data.json · build 57 · 2026-09-11 · public render. Do not hand-edit the HTML deck; it regenerates from the same file.</t>
         </is>
       </c>
     </row>
@@ -33585,7 +33585,7 @@
     <row r="284">
       <c r="A284" s="17" t="inlineStr">
         <is>
-          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 56, 2026-09-11.</t>
+          <t>NOTE. A filled LinkedIn cell means the profile was opened or the search result read and the headline named the firm; column W records what was read. Where that test failed the cell is left empty rather than guessed, because a fabricated slug passes visual inspection and then fails in front of the person it names. Column Q searches for the empty ones in your own session. Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Capital is a qualifier, not a count. Source: ICON Greater Houston screen, build 57, 2026-09-11.</t>
         </is>
       </c>
     </row>

</xml_diff>